<commit_message>
Lens: axis labels on phones, and the dogs on the 2021 ring
Phones get their axis labels back, just fewer and smaller:
- About: years run up the vertical axis.
- Engineering: scale ticks under the plot; complexity labels just
  inside it.
- Projects: every fourth year.
- Travel: every 30° of longitude and latitude.
The x axis titles move above the plot on phones, clear of the ticks.

Jaylee and Helga now sit on About's 2021 ring instead of beside the
quiet line. They take the clearest flat stretch of the ring, and their
names show on hover.

Art keeps its axis names readable (marks are pushed off them), and on
phones the film stacks are captioned with a short name.

CLAUDE.md and the workbook record the dogs' new spot, and that phones
keep their labels.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KQRhL2ffDZuAUo4d7ziJty
</commit_message>
<xml_diff>
--- a/planning/site-artifacts.xlsx
+++ b/planning/site-artifacts.xlsx
@@ -88,7 +88,7 @@
     <t xml:space="preserve">Keep it uncluttered: personal context supports the work quietly, it never crowds it.</t>
   </si>
   <si>
-    <t xml:space="preserve">Latest decisions: one quiet line in About ("Based in Austin · English, Italian, learning Portuguese"), with Jaylee and Helga as one small sprite each beside it, not in the orbit. No languages on the Travel map; no sports on films or trips. The Travel map is small dots (lived, photos, worked), lines only for the moves between places lived, and the countries visited shaded.</t>
+    <t xml:space="preserve">Latest decisions: one quiet line in About ("Based in Austin · English, Italian, learning Portuguese"), with Jaylee and Helga as one small sprite each sitting on the 2021 ring (not a tile). No languages on the Travel map; no sports on films or trips. The Travel map is small dots (lived, photos, worked), lines only for the moves between places lived, and the countries visited shaded.</t>
   </si>
   <si>
     <t xml:space="preserve">Sheets</t>
@@ -1894,7 +1894,7 @@
     <t xml:space="preserve">Jaylee and Helga</t>
   </si>
   <si>
-    <t xml:space="preserve">Named, as one small sprite of each beside the quiet line in About (not in the orbit).</t>
+    <t xml:space="preserve">Named, as one small sprite of each sitting on the 2021 ring in About (name on hover), never as a tile.</t>
   </si>
   <si>
     <t xml:space="preserve">not sure how to diplay all the about profle stuff don’t want to make everythign to busy also!!</t>

</xml_diff>

<commit_message>
Lens Travel: zoom and pan, worked-at-home marks, born marker
The map can now be zoomed and panned: wheel or trackpad pinch,
touch pinch, drag, double-click, and + / − / fit buttons. It always
opens on the whole fitted view. Land and the visited countries are
drawn once in degrees and moved with a transform, so zooming only
redraws the grid, the lines and the labels. Finer 50m coastlines load
the first time the map is zoomed in close. Dots beyond the view step
out, and labels are placed again for each view.

Homes where Grant also worked (Chicago, Milan, Dallas, Austin) are
framed in the "worked" square. Wilmette gets a "born" ring and
"born · until 2014". On phones its label reads "Chicago · born" and
the later Chicago dot goes unlabelled.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KQRhL2ffDZuAUo4d7ziJty
</commit_message>
<xml_diff>
--- a/planning/site-artifacts.xlsx
+++ b/planning/site-artifacts.xlsx
@@ -88,7 +88,7 @@
     <t xml:space="preserve">Keep it uncluttered: personal context supports the work quietly, it never crowds it.</t>
   </si>
   <si>
-    <t xml:space="preserve">Latest decisions: one quiet line in About ("Based in Austin · English, Italian, learning Portuguese"), with Jaylee and Helga as one small sprite each sitting on the 2021 ring (not a tile). No languages on the Travel map; no sports on films or trips. The Travel map is small dots (lived, photos, worked), lines only for the moves between places lived, and the countries visited shaded.</t>
+    <t xml:space="preserve">Latest decisions: one quiet line in About ("Based in Austin · English, Italian, learning Portuguese"), with Jaylee and Helga as one small sprite each sitting on the 2021 ring (not a tile). No languages on the Travel map; no sports on films or trips. The Travel map is small dots (lived, photos, worked; homes you also worked in get the worked square, Wilmette is marked born), lines only for the moves between places lived, the countries visited shaded, and it zooms and pans.</t>
   </si>
   <si>
     <t xml:space="preserve">Sheets</t>
@@ -1450,7 +1450,7 @@
     <t xml:space="preserve">USA</t>
   </si>
   <si>
-    <t xml:space="preserve">Confirmed: before Lawrence</t>
+    <t xml:space="preserve">Confirmed: before Lawrence. Marked "born" on the map (phones say "Chicago · born")</t>
   </si>
   <si>
     <t xml:space="preserve">Confirmed</t>

</xml_diff>

<commit_message>
Lens Apps: add the factory digital twin
A new featured app, "Factory digital twin", sits in Apps with a
generated placeholder: an isometric factory floor with machines, a
conveyor and live status tags. Grant hasn't given the details yet, so
the wording is general. The year, the "Personal" tag and the missing
link are placeholders.

The workbook gets it as A14 (Apps ●, Featured Yes), plus open
question #22 asking what it models, what it's built with, when, links
or screenshots, and whether it's tied to an employer. Apps now has 7
featured items against a suggested maximum of 6, so the Section
summary flags "Trim".

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KQRhL2ffDZuAUo4d7ziJty
</commit_message>
<xml_diff>
--- a/planning/site-artifacts.xlsx
+++ b/planning/site-artifacts.xlsx
@@ -18,7 +18,7 @@
     <sheet name="Open questions" sheetId="8" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Artifacts!$A$1:$W$64</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Artifacts!$A$1:$W$65</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1502" uniqueCount="669">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1516" uniqueCount="679">
   <si>
     <t xml:space="preserve">Site artifacts: mapping workbook</t>
   </si>
@@ -1138,6 +1138,30 @@
     <t xml:space="preserve">Python, Llama 3.x, fine-tuning, quantization, web scraping</t>
   </si>
   <si>
+    <t xml:space="preserve">A14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Factory digital twin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Personal (verify)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Digital twin of a factory (details to come).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Screen with real screenshot / 3D view</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maybe (it is a model)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What it models, tech, year, link, screenshots. Personal, or tied to an employer (confidential)?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Your note in chat</t>
+  </si>
+  <si>
     <t xml:space="preserve">Films (35mm albums)</t>
   </si>
   <si>
@@ -2075,6 +2099,12 @@
   </si>
   <si>
     <t xml:space="preserve">$10M is fine: reverted to &gt;$10M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Factory digital twin (A14): what does it model, what is it built with, when, is there a link or screenshots, and is it personal or tied to an employer?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A14, Apps</t>
   </si>
 </sst>
 </file>
@@ -2981,7 +3011,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:W64"/>
+  <dimension ref="A1:W65"/>
   <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6"/>
@@ -5452,107 +5482,97 @@
         <v>281</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="13" t="s">
+    <row r="46" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="15" t="s">
         <v>356</v>
       </c>
-      <c r="B46" s="14"/>
-      <c r="C46" s="14"/>
-      <c r="D46" s="14"/>
-      <c r="E46" s="14"/>
-      <c r="F46" s="14"/>
-      <c r="G46" s="14"/>
-      <c r="H46" s="14"/>
-      <c r="I46" s="14"/>
-      <c r="J46" s="14"/>
-      <c r="K46" s="14"/>
-      <c r="L46" s="14"/>
-      <c r="M46" s="14"/>
-      <c r="N46" s="14"/>
-      <c r="O46" s="14"/>
-      <c r="P46" s="14"/>
-      <c r="Q46" s="14"/>
-      <c r="R46" s="14"/>
-      <c r="S46" s="14"/>
-      <c r="T46" s="14"/>
-      <c r="U46" s="14"/>
-      <c r="V46" s="14"/>
-      <c r="W46" s="14"/>
-    </row>
-    <row r="47" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="15" t="s">
+      <c r="B46" s="16" t="s">
         <v>357</v>
       </c>
-      <c r="B47" s="16" t="s">
+      <c r="C46" s="17" t="s">
+        <v>271</v>
+      </c>
+      <c r="D46" s="17" t="s">
         <v>358</v>
       </c>
-      <c r="C47" s="17" t="s">
+      <c r="E46" s="17"/>
+      <c r="F46" s="15"/>
+      <c r="G46" s="15"/>
+      <c r="H46" s="17" t="s">
         <v>359</v>
       </c>
-      <c r="D47" s="17" t="s">
+      <c r="I46" s="17"/>
+      <c r="J46" s="17"/>
+      <c r="K46" s="17"/>
+      <c r="L46" s="20"/>
+      <c r="M46" s="19"/>
+      <c r="N46" s="20"/>
+      <c r="O46" s="20"/>
+      <c r="P46" s="20"/>
+      <c r="Q46" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="R46" s="20" t="s">
+        <v>60</v>
+      </c>
+      <c r="S46" s="17" t="s">
         <v>360</v>
       </c>
-      <c r="E47" s="17" t="s">
+      <c r="T46" s="17" t="s">
         <v>361</v>
       </c>
-      <c r="F47" s="15" t="n">
-        <v>2026</v>
-      </c>
-      <c r="G47" s="15" t="n">
-        <v>2026</v>
-      </c>
-      <c r="H47" s="17" t="s">
+      <c r="U46" s="17" t="s">
+        <v>63</v>
+      </c>
+      <c r="V46" s="21" t="s">
         <v>362</v>
       </c>
-      <c r="I47" s="17"/>
-      <c r="J47" s="17" t="s">
-        <v>360</v>
-      </c>
-      <c r="K47" s="17"/>
-      <c r="L47" s="20"/>
-      <c r="M47" s="20"/>
-      <c r="N47" s="20"/>
-      <c r="O47" s="25" t="s">
-        <v>58</v>
-      </c>
-      <c r="P47" s="22" t="s">
-        <v>59</v>
-      </c>
-      <c r="Q47" s="20"/>
-      <c r="R47" s="20" t="s">
-        <v>60</v>
-      </c>
-      <c r="S47" s="17" t="s">
+      <c r="W46" s="17" t="s">
         <v>363</v>
       </c>
-      <c r="T47" s="17" t="s">
+    </row>
+    <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="13" t="s">
         <v>364</v>
       </c>
-      <c r="U47" s="17" t="s">
+      <c r="B47" s="14"/>
+      <c r="C47" s="14"/>
+      <c r="D47" s="14"/>
+      <c r="E47" s="14"/>
+      <c r="F47" s="14"/>
+      <c r="G47" s="14"/>
+      <c r="H47" s="14"/>
+      <c r="I47" s="14"/>
+      <c r="J47" s="14"/>
+      <c r="K47" s="14"/>
+      <c r="L47" s="14"/>
+      <c r="M47" s="14"/>
+      <c r="N47" s="14"/>
+      <c r="O47" s="14"/>
+      <c r="P47" s="14"/>
+      <c r="Q47" s="14"/>
+      <c r="R47" s="14"/>
+      <c r="S47" s="14"/>
+      <c r="T47" s="14"/>
+      <c r="U47" s="14"/>
+      <c r="V47" s="14"/>
+      <c r="W47" s="14"/>
+    </row>
+    <row r="48" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="15" t="s">
         <v>365</v>
       </c>
-      <c r="V47" s="21" t="s">
+      <c r="B48" s="16" t="s">
         <v>366</v>
       </c>
-      <c r="W47" s="17" t="s">
+      <c r="C48" s="17" t="s">
         <v>367</v>
       </c>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="15" t="s">
+      <c r="D48" s="17" t="s">
         <v>368</v>
       </c>
-      <c r="B48" s="16" t="s">
+      <c r="E48" s="17" t="s">
         <v>369</v>
-      </c>
-      <c r="C48" s="17" t="s">
-        <v>359</v>
-      </c>
-      <c r="D48" s="17" t="s">
-        <v>360</v>
-      </c>
-      <c r="E48" s="17" t="s">
-        <v>370</v>
       </c>
       <c r="F48" s="15" t="n">
         <v>2026</v>
@@ -5561,11 +5581,11 @@
         <v>2026</v>
       </c>
       <c r="H48" s="17" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="I48" s="17"/>
       <c r="J48" s="17" t="s">
-        <v>360</v>
+        <v>368</v>
       </c>
       <c r="K48" s="17"/>
       <c r="L48" s="20"/>
@@ -5582,49 +5602,49 @@
         <v>60</v>
       </c>
       <c r="S48" s="17" t="s">
-        <v>363</v>
+        <v>371</v>
       </c>
       <c r="T48" s="17" t="s">
-        <v>364</v>
+        <v>372</v>
       </c>
       <c r="U48" s="17" t="s">
-        <v>365</v>
+        <v>373</v>
       </c>
       <c r="V48" s="21" t="s">
-        <v>366</v>
+        <v>374</v>
       </c>
       <c r="W48" s="17" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="15" t="s">
+        <v>376</v>
+      </c>
+      <c r="B49" s="16" t="s">
+        <v>377</v>
+      </c>
+      <c r="C49" s="17" t="s">
         <v>367</v>
       </c>
-    </row>
-    <row r="49" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="15" t="s">
-        <v>372</v>
-      </c>
-      <c r="B49" s="16" t="s">
-        <v>373</v>
-      </c>
-      <c r="C49" s="17" t="s">
-        <v>359</v>
-      </c>
       <c r="D49" s="17" t="s">
-        <v>360</v>
+        <v>368</v>
       </c>
       <c r="E49" s="17" t="s">
-        <v>374</v>
-      </c>
-      <c r="F49" s="15" t="s">
-        <v>53</v>
-      </c>
-      <c r="G49" s="15" t="s">
-        <v>53</v>
+        <v>378</v>
+      </c>
+      <c r="F49" s="15" t="n">
+        <v>2026</v>
+      </c>
+      <c r="G49" s="15" t="n">
+        <v>2026</v>
       </c>
       <c r="H49" s="17" t="s">
-        <v>375</v>
+        <v>379</v>
       </c>
       <c r="I49" s="17"/>
       <c r="J49" s="17" t="s">
-        <v>360</v>
+        <v>368</v>
       </c>
       <c r="K49" s="17"/>
       <c r="L49" s="20"/>
@@ -5641,36 +5661,36 @@
         <v>60</v>
       </c>
       <c r="S49" s="17" t="s">
-        <v>363</v>
+        <v>371</v>
       </c>
       <c r="T49" s="17" t="s">
-        <v>364</v>
+        <v>372</v>
       </c>
       <c r="U49" s="17" t="s">
-        <v>365</v>
+        <v>373</v>
       </c>
       <c r="V49" s="21" t="s">
-        <v>366</v>
+        <v>374</v>
       </c>
       <c r="W49" s="17" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="15" t="s">
+        <v>380</v>
+      </c>
+      <c r="B50" s="16" t="s">
+        <v>381</v>
+      </c>
+      <c r="C50" s="17" t="s">
         <v>367</v>
       </c>
-    </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="15" t="s">
-        <v>376</v>
-      </c>
-      <c r="B50" s="16" t="s">
-        <v>377</v>
-      </c>
-      <c r="C50" s="17" t="s">
-        <v>359</v>
-      </c>
       <c r="D50" s="17" t="s">
-        <v>360</v>
+        <v>368</v>
       </c>
       <c r="E50" s="17" t="s">
-        <v>378</v>
+        <v>382</v>
       </c>
       <c r="F50" s="15" t="s">
         <v>53</v>
@@ -5679,11 +5699,11 @@
         <v>53</v>
       </c>
       <c r="H50" s="17" t="s">
-        <v>379</v>
+        <v>383</v>
       </c>
       <c r="I50" s="17"/>
       <c r="J50" s="17" t="s">
-        <v>360</v>
+        <v>368</v>
       </c>
       <c r="K50" s="17"/>
       <c r="L50" s="20"/>
@@ -5700,36 +5720,36 @@
         <v>60</v>
       </c>
       <c r="S50" s="17" t="s">
-        <v>363</v>
+        <v>371</v>
       </c>
       <c r="T50" s="17" t="s">
-        <v>364</v>
+        <v>372</v>
       </c>
       <c r="U50" s="17" t="s">
-        <v>365</v>
+        <v>373</v>
       </c>
       <c r="V50" s="21" t="s">
-        <v>366</v>
+        <v>374</v>
       </c>
       <c r="W50" s="17" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="15" t="s">
+        <v>384</v>
+      </c>
+      <c r="B51" s="16" t="s">
+        <v>385</v>
+      </c>
+      <c r="C51" s="17" t="s">
         <v>367</v>
       </c>
-    </row>
-    <row r="51" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="15" t="s">
-        <v>380</v>
-      </c>
-      <c r="B51" s="16" t="s">
-        <v>381</v>
-      </c>
-      <c r="C51" s="17" t="s">
-        <v>359</v>
-      </c>
       <c r="D51" s="17" t="s">
-        <v>360</v>
+        <v>368</v>
       </c>
       <c r="E51" s="17" t="s">
-        <v>382</v>
+        <v>386</v>
       </c>
       <c r="F51" s="15" t="s">
         <v>53</v>
@@ -5738,16 +5758,14 @@
         <v>53</v>
       </c>
       <c r="H51" s="17" t="s">
-        <v>383</v>
+        <v>387</v>
       </c>
       <c r="I51" s="17"/>
       <c r="J51" s="17" t="s">
-        <v>360</v>
+        <v>368</v>
       </c>
       <c r="K51" s="17"/>
-      <c r="L51" s="18" t="s">
-        <v>59</v>
-      </c>
+      <c r="L51" s="20"/>
       <c r="M51" s="20"/>
       <c r="N51" s="20"/>
       <c r="O51" s="25" t="s">
@@ -5761,52 +5779,54 @@
         <v>60</v>
       </c>
       <c r="S51" s="17" t="s">
-        <v>363</v>
+        <v>371</v>
       </c>
       <c r="T51" s="17" t="s">
-        <v>364</v>
+        <v>372</v>
       </c>
       <c r="U51" s="17" t="s">
-        <v>365</v>
+        <v>373</v>
       </c>
       <c r="V51" s="21" t="s">
-        <v>366</v>
+        <v>374</v>
       </c>
       <c r="W51" s="17" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="15" t="s">
+        <v>388</v>
+      </c>
+      <c r="B52" s="16" t="s">
+        <v>389</v>
+      </c>
+      <c r="C52" s="17" t="s">
         <v>367</v>
       </c>
-    </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A52" s="15" t="s">
-        <v>384</v>
-      </c>
-      <c r="B52" s="16" t="s">
-        <v>385</v>
-      </c>
-      <c r="C52" s="17" t="s">
-        <v>359</v>
-      </c>
       <c r="D52" s="17" t="s">
-        <v>360</v>
+        <v>368</v>
       </c>
       <c r="E52" s="17" t="s">
-        <v>386</v>
-      </c>
-      <c r="F52" s="15" t="n">
-        <v>2024</v>
-      </c>
-      <c r="G52" s="15" t="n">
-        <v>2024</v>
+        <v>390</v>
+      </c>
+      <c r="F52" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="G52" s="15" t="s">
+        <v>53</v>
       </c>
       <c r="H52" s="17" t="s">
-        <v>387</v>
+        <v>391</v>
       </c>
       <c r="I52" s="17"/>
       <c r="J52" s="17" t="s">
-        <v>360</v>
+        <v>368</v>
       </c>
       <c r="K52" s="17"/>
-      <c r="L52" s="20"/>
+      <c r="L52" s="18" t="s">
+        <v>59</v>
+      </c>
       <c r="M52" s="20"/>
       <c r="N52" s="20"/>
       <c r="O52" s="25" t="s">
@@ -5820,49 +5840,49 @@
         <v>60</v>
       </c>
       <c r="S52" s="17" t="s">
-        <v>363</v>
+        <v>371</v>
       </c>
       <c r="T52" s="17" t="s">
-        <v>364</v>
+        <v>372</v>
       </c>
       <c r="U52" s="17" t="s">
-        <v>365</v>
+        <v>373</v>
       </c>
       <c r="V52" s="21" t="s">
-        <v>366</v>
+        <v>374</v>
       </c>
       <c r="W52" s="17" t="s">
-        <v>367</v>
+        <v>375</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="15" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
       <c r="B53" s="16" t="s">
-        <v>389</v>
+        <v>393</v>
       </c>
       <c r="C53" s="17" t="s">
-        <v>359</v>
+        <v>367</v>
       </c>
       <c r="D53" s="17" t="s">
-        <v>360</v>
+        <v>368</v>
       </c>
       <c r="E53" s="17" t="s">
-        <v>390</v>
+        <v>394</v>
       </c>
       <c r="F53" s="15" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="G53" s="15" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="H53" s="17" t="s">
-        <v>391</v>
+        <v>395</v>
       </c>
       <c r="I53" s="17"/>
       <c r="J53" s="17" t="s">
-        <v>360</v>
+        <v>368</v>
       </c>
       <c r="K53" s="17"/>
       <c r="L53" s="20"/>
@@ -5879,36 +5899,36 @@
         <v>60</v>
       </c>
       <c r="S53" s="17" t="s">
-        <v>363</v>
+        <v>371</v>
       </c>
       <c r="T53" s="17" t="s">
-        <v>364</v>
+        <v>372</v>
       </c>
       <c r="U53" s="17" t="s">
-        <v>365</v>
+        <v>373</v>
       </c>
       <c r="V53" s="21" t="s">
-        <v>366</v>
+        <v>374</v>
       </c>
       <c r="W53" s="17" t="s">
-        <v>367</v>
+        <v>375</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="15" t="s">
-        <v>392</v>
+        <v>396</v>
       </c>
       <c r="B54" s="16" t="s">
-        <v>393</v>
+        <v>397</v>
       </c>
       <c r="C54" s="17" t="s">
-        <v>359</v>
+        <v>367</v>
       </c>
       <c r="D54" s="17" t="s">
-        <v>360</v>
+        <v>368</v>
       </c>
       <c r="E54" s="17" t="s">
-        <v>394</v>
+        <v>398</v>
       </c>
       <c r="F54" s="15" t="n">
         <v>2023</v>
@@ -5917,11 +5937,11 @@
         <v>2023</v>
       </c>
       <c r="H54" s="17" t="s">
-        <v>383</v>
+        <v>399</v>
       </c>
       <c r="I54" s="17"/>
       <c r="J54" s="17" t="s">
-        <v>360</v>
+        <v>368</v>
       </c>
       <c r="K54" s="17"/>
       <c r="L54" s="20"/>
@@ -5938,49 +5958,49 @@
         <v>60</v>
       </c>
       <c r="S54" s="17" t="s">
-        <v>363</v>
+        <v>371</v>
       </c>
       <c r="T54" s="17" t="s">
-        <v>364</v>
+        <v>372</v>
       </c>
       <c r="U54" s="17" t="s">
-        <v>365</v>
+        <v>373</v>
       </c>
       <c r="V54" s="21" t="s">
-        <v>366</v>
+        <v>374</v>
       </c>
       <c r="W54" s="17" t="s">
-        <v>367</v>
+        <v>375</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="15" t="s">
-        <v>395</v>
+        <v>400</v>
       </c>
       <c r="B55" s="16" t="s">
-        <v>396</v>
+        <v>401</v>
       </c>
       <c r="C55" s="17" t="s">
-        <v>359</v>
+        <v>367</v>
       </c>
       <c r="D55" s="17" t="s">
-        <v>360</v>
+        <v>368</v>
       </c>
       <c r="E55" s="17" t="s">
-        <v>378</v>
+        <v>402</v>
       </c>
       <c r="F55" s="15" t="n">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="G55" s="15" t="n">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="H55" s="17" t="s">
-        <v>397</v>
+        <v>391</v>
       </c>
       <c r="I55" s="17"/>
       <c r="J55" s="17" t="s">
-        <v>360</v>
+        <v>368</v>
       </c>
       <c r="K55" s="17"/>
       <c r="L55" s="20"/>
@@ -5997,49 +6017,49 @@
         <v>60</v>
       </c>
       <c r="S55" s="17" t="s">
-        <v>363</v>
+        <v>371</v>
       </c>
       <c r="T55" s="17" t="s">
-        <v>364</v>
+        <v>372</v>
       </c>
       <c r="U55" s="17" t="s">
-        <v>365</v>
+        <v>373</v>
       </c>
       <c r="V55" s="21" t="s">
-        <v>366</v>
+        <v>374</v>
       </c>
       <c r="W55" s="17" t="s">
-        <v>367</v>
+        <v>375</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="15" t="s">
-        <v>398</v>
+        <v>403</v>
       </c>
       <c r="B56" s="16" t="s">
-        <v>399</v>
+        <v>404</v>
       </c>
       <c r="C56" s="17" t="s">
-        <v>359</v>
+        <v>367</v>
       </c>
       <c r="D56" s="17" t="s">
-        <v>360</v>
+        <v>368</v>
       </c>
       <c r="E56" s="17" t="s">
-        <v>400</v>
+        <v>386</v>
       </c>
       <c r="F56" s="15" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="G56" s="15" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="H56" s="17" t="s">
-        <v>397</v>
+        <v>405</v>
       </c>
       <c r="I56" s="17"/>
       <c r="J56" s="17" t="s">
-        <v>360</v>
+        <v>368</v>
       </c>
       <c r="K56" s="17"/>
       <c r="L56" s="20"/>
@@ -6056,49 +6076,49 @@
         <v>60</v>
       </c>
       <c r="S56" s="17" t="s">
-        <v>363</v>
+        <v>371</v>
       </c>
       <c r="T56" s="17" t="s">
-        <v>364</v>
+        <v>372</v>
       </c>
       <c r="U56" s="17" t="s">
-        <v>365</v>
+        <v>373</v>
       </c>
       <c r="V56" s="21" t="s">
-        <v>366</v>
+        <v>374</v>
       </c>
       <c r="W56" s="17" t="s">
-        <v>367</v>
+        <v>375</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="15" t="s">
-        <v>401</v>
+        <v>406</v>
       </c>
       <c r="B57" s="16" t="s">
-        <v>402</v>
+        <v>407</v>
       </c>
       <c r="C57" s="17" t="s">
-        <v>359</v>
+        <v>367</v>
       </c>
       <c r="D57" s="17" t="s">
-        <v>360</v>
+        <v>368</v>
       </c>
       <c r="E57" s="17" t="s">
-        <v>403</v>
+        <v>408</v>
       </c>
       <c r="F57" s="15" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="G57" s="15" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="H57" s="17" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="I57" s="17"/>
       <c r="J57" s="17" t="s">
-        <v>360</v>
+        <v>368</v>
       </c>
       <c r="K57" s="17"/>
       <c r="L57" s="20"/>
@@ -6115,121 +6135,125 @@
         <v>60</v>
       </c>
       <c r="S57" s="17" t="s">
-        <v>363</v>
+        <v>371</v>
       </c>
       <c r="T57" s="17" t="s">
-        <v>364</v>
+        <v>372</v>
       </c>
       <c r="U57" s="17" t="s">
-        <v>365</v>
-      </c>
-      <c r="V57" s="21"/>
+        <v>373</v>
+      </c>
+      <c r="V57" s="21" t="s">
+        <v>374</v>
+      </c>
       <c r="W57" s="17" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A58" s="15" t="s">
+        <v>409</v>
+      </c>
+      <c r="B58" s="16" t="s">
+        <v>410</v>
+      </c>
+      <c r="C58" s="17" t="s">
         <v>367</v>
       </c>
-    </row>
-    <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="13" t="s">
-        <v>405</v>
-      </c>
-      <c r="B58" s="14"/>
-      <c r="C58" s="14"/>
-      <c r="D58" s="14"/>
-      <c r="E58" s="14"/>
-      <c r="F58" s="14"/>
-      <c r="G58" s="14"/>
-      <c r="H58" s="14"/>
-      <c r="I58" s="14"/>
-      <c r="J58" s="14"/>
-      <c r="K58" s="14"/>
-      <c r="L58" s="14"/>
-      <c r="M58" s="14"/>
-      <c r="N58" s="14"/>
-      <c r="O58" s="14"/>
-      <c r="P58" s="14"/>
-      <c r="Q58" s="14"/>
-      <c r="R58" s="14"/>
-      <c r="S58" s="14"/>
-      <c r="T58" s="14"/>
-      <c r="U58" s="14"/>
-      <c r="V58" s="14"/>
-      <c r="W58" s="14"/>
-    </row>
-    <row r="59" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="15" t="s">
-        <v>406</v>
-      </c>
-      <c r="B59" s="16" t="s">
-        <v>407</v>
-      </c>
-      <c r="C59" s="17" t="s">
-        <v>408</v>
-      </c>
-      <c r="D59" s="17" t="s">
-        <v>409</v>
-      </c>
-      <c r="E59" s="17" t="s">
-        <v>407</v>
-      </c>
-      <c r="F59" s="15"/>
-      <c r="G59" s="15"/>
-      <c r="H59" s="17" t="s">
-        <v>410</v>
-      </c>
-      <c r="I59" s="17"/>
-      <c r="J59" s="17"/>
-      <c r="K59" s="17"/>
-      <c r="L59" s="18" t="s">
+      <c r="D58" s="17" t="s">
+        <v>368</v>
+      </c>
+      <c r="E58" s="17" t="s">
+        <v>411</v>
+      </c>
+      <c r="F58" s="15" t="n">
+        <v>2022</v>
+      </c>
+      <c r="G58" s="15" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H58" s="17" t="s">
+        <v>412</v>
+      </c>
+      <c r="I58" s="17"/>
+      <c r="J58" s="17" t="s">
+        <v>368</v>
+      </c>
+      <c r="K58" s="17"/>
+      <c r="L58" s="20"/>
+      <c r="M58" s="20"/>
+      <c r="N58" s="20"/>
+      <c r="O58" s="25" t="s">
+        <v>58</v>
+      </c>
+      <c r="P58" s="22" t="s">
         <v>59</v>
       </c>
-      <c r="M59" s="20"/>
-      <c r="N59" s="20"/>
-      <c r="O59" s="20"/>
-      <c r="P59" s="22" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q59" s="20"/>
-      <c r="R59" s="20" t="s">
+      <c r="Q58" s="20"/>
+      <c r="R58" s="20" t="s">
         <v>60</v>
       </c>
-      <c r="S59" s="17" t="s">
-        <v>411</v>
-      </c>
-      <c r="T59" s="17" t="s">
-        <v>62</v>
-      </c>
-      <c r="U59" s="17"/>
-      <c r="V59" s="21" t="s">
-        <v>412</v>
-      </c>
-      <c r="W59" s="17" t="s">
+      <c r="S58" s="17" t="s">
+        <v>371</v>
+      </c>
+      <c r="T58" s="17" t="s">
+        <v>372</v>
+      </c>
+      <c r="U58" s="17" t="s">
+        <v>373</v>
+      </c>
+      <c r="V58" s="21"/>
+      <c r="W58" s="17" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="13" t="s">
         <v>413</v>
       </c>
+      <c r="B59" s="14"/>
+      <c r="C59" s="14"/>
+      <c r="D59" s="14"/>
+      <c r="E59" s="14"/>
+      <c r="F59" s="14"/>
+      <c r="G59" s="14"/>
+      <c r="H59" s="14"/>
+      <c r="I59" s="14"/>
+      <c r="J59" s="14"/>
+      <c r="K59" s="14"/>
+      <c r="L59" s="14"/>
+      <c r="M59" s="14"/>
+      <c r="N59" s="14"/>
+      <c r="O59" s="14"/>
+      <c r="P59" s="14"/>
+      <c r="Q59" s="14"/>
+      <c r="R59" s="14"/>
+      <c r="S59" s="14"/>
+      <c r="T59" s="14"/>
+      <c r="U59" s="14"/>
+      <c r="V59" s="14"/>
+      <c r="W59" s="14"/>
     </row>
     <row r="60" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="15" t="s">
         <v>414</v>
       </c>
       <c r="B60" s="16" t="s">
-        <v>104</v>
+        <v>415</v>
       </c>
       <c r="C60" s="17" t="s">
-        <v>408</v>
+        <v>416</v>
       </c>
       <c r="D60" s="17" t="s">
+        <v>417</v>
+      </c>
+      <c r="E60" s="17" t="s">
         <v>415</v>
       </c>
-      <c r="E60" s="17" t="s">
-        <v>104</v>
-      </c>
-      <c r="F60" s="15" t="s">
-        <v>105</v>
-      </c>
-      <c r="G60" s="15" t="s">
-        <v>88</v>
-      </c>
+      <c r="F60" s="15"/>
+      <c r="G60" s="15"/>
       <c r="H60" s="17" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="I60" s="17"/>
       <c r="J60" s="17"/>
@@ -6248,43 +6272,43 @@
         <v>60</v>
       </c>
       <c r="S60" s="17" t="s">
-        <v>411</v>
+        <v>419</v>
       </c>
       <c r="T60" s="17" t="s">
         <v>62</v>
       </c>
       <c r="U60" s="17"/>
       <c r="V60" s="21" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="W60" s="17" t="s">
-        <v>413</v>
+        <v>421</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="15" t="s">
-        <v>418</v>
+        <v>422</v>
       </c>
       <c r="B61" s="16" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="C61" s="17" t="s">
-        <v>408</v>
+        <v>416</v>
       </c>
       <c r="D61" s="17" t="s">
-        <v>419</v>
+        <v>423</v>
       </c>
       <c r="E61" s="17" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="F61" s="15" t="s">
+        <v>105</v>
+      </c>
+      <c r="G61" s="15" t="s">
         <v>88</v>
       </c>
-      <c r="G61" s="15" t="s">
-        <v>80</v>
-      </c>
       <c r="H61" s="17" t="s">
-        <v>420</v>
+        <v>424</v>
       </c>
       <c r="I61" s="17"/>
       <c r="J61" s="17"/>
@@ -6303,43 +6327,43 @@
         <v>60</v>
       </c>
       <c r="S61" s="17" t="s">
-        <v>411</v>
+        <v>419</v>
       </c>
       <c r="T61" s="17" t="s">
         <v>62</v>
       </c>
       <c r="U61" s="17"/>
       <c r="V61" s="21" t="s">
+        <v>425</v>
+      </c>
+      <c r="W61" s="17" t="s">
         <v>421</v>
-      </c>
-      <c r="W61" s="17" t="s">
-        <v>413</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="15" t="s">
-        <v>422</v>
+        <v>426</v>
       </c>
       <c r="B62" s="16" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="C62" s="17" t="s">
-        <v>408</v>
+        <v>416</v>
       </c>
       <c r="D62" s="17" t="s">
-        <v>423</v>
+        <v>427</v>
       </c>
       <c r="E62" s="17" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="F62" s="15" t="s">
+        <v>88</v>
+      </c>
+      <c r="G62" s="15" t="s">
         <v>80</v>
       </c>
-      <c r="G62" s="15" t="s">
-        <v>70</v>
-      </c>
       <c r="H62" s="17" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="I62" s="17"/>
       <c r="J62" s="17"/>
@@ -6358,43 +6382,43 @@
         <v>60</v>
       </c>
       <c r="S62" s="17" t="s">
-        <v>411</v>
+        <v>419</v>
       </c>
       <c r="T62" s="17" t="s">
         <v>62</v>
       </c>
       <c r="U62" s="17"/>
       <c r="V62" s="21" t="s">
-        <v>425</v>
+        <v>429</v>
       </c>
       <c r="W62" s="17" t="s">
-        <v>413</v>
+        <v>421</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="15" t="s">
-        <v>426</v>
+        <v>430</v>
       </c>
       <c r="B63" s="16" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="C63" s="17" t="s">
-        <v>408</v>
+        <v>416</v>
       </c>
       <c r="D63" s="17" t="s">
-        <v>427</v>
+        <v>431</v>
       </c>
       <c r="E63" s="17" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="F63" s="15" t="s">
+        <v>80</v>
+      </c>
+      <c r="G63" s="15" t="s">
         <v>70</v>
       </c>
-      <c r="G63" s="15" t="s">
-        <v>71</v>
-      </c>
       <c r="H63" s="17" t="s">
-        <v>428</v>
+        <v>432</v>
       </c>
       <c r="I63" s="17"/>
       <c r="J63" s="17"/>
@@ -6413,43 +6437,43 @@
         <v>60</v>
       </c>
       <c r="S63" s="17" t="s">
-        <v>411</v>
+        <v>419</v>
       </c>
       <c r="T63" s="17" t="s">
         <v>62</v>
       </c>
       <c r="U63" s="17"/>
       <c r="V63" s="21" t="s">
-        <v>429</v>
+        <v>433</v>
       </c>
       <c r="W63" s="17" t="s">
-        <v>413</v>
+        <v>421</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="15" t="s">
-        <v>430</v>
+        <v>434</v>
       </c>
       <c r="B64" s="16" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="C64" s="17" t="s">
-        <v>408</v>
+        <v>416</v>
       </c>
       <c r="D64" s="17" t="s">
-        <v>431</v>
+        <v>435</v>
       </c>
       <c r="E64" s="17" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="F64" s="15" t="s">
-        <v>53</v>
+        <v>70</v>
       </c>
       <c r="G64" s="15" t="s">
-        <v>54</v>
+        <v>71</v>
       </c>
       <c r="H64" s="17" t="s">
-        <v>432</v>
+        <v>436</v>
       </c>
       <c r="I64" s="17"/>
       <c r="J64" s="17"/>
@@ -6468,21 +6492,76 @@
         <v>60</v>
       </c>
       <c r="S64" s="17" t="s">
-        <v>411</v>
+        <v>419</v>
       </c>
       <c r="T64" s="17" t="s">
         <v>62</v>
       </c>
       <c r="U64" s="17"/>
       <c r="V64" s="21" t="s">
-        <v>433</v>
+        <v>437</v>
       </c>
       <c r="W64" s="17" t="s">
-        <v>413</v>
+        <v>421</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A65" s="15" t="s">
+        <v>438</v>
+      </c>
+      <c r="B65" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="C65" s="17" t="s">
+        <v>416</v>
+      </c>
+      <c r="D65" s="17" t="s">
+        <v>439</v>
+      </c>
+      <c r="E65" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="F65" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="G65" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="H65" s="17" t="s">
+        <v>440</v>
+      </c>
+      <c r="I65" s="17"/>
+      <c r="J65" s="17"/>
+      <c r="K65" s="17"/>
+      <c r="L65" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="M65" s="20"/>
+      <c r="N65" s="20"/>
+      <c r="O65" s="20"/>
+      <c r="P65" s="22" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q65" s="20"/>
+      <c r="R65" s="20" t="s">
+        <v>60</v>
+      </c>
+      <c r="S65" s="17" t="s">
+        <v>419</v>
+      </c>
+      <c r="T65" s="17" t="s">
+        <v>62</v>
+      </c>
+      <c r="U65" s="17"/>
+      <c r="V65" s="21" t="s">
+        <v>441</v>
+      </c>
+      <c r="W65" s="17" t="s">
+        <v>421</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:W64"/>
+  <autoFilter ref="A1:W65"/>
   <dataValidations count="2">
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="L2:Q124" type="list">
       <formula1>"●,○"</formula1>
@@ -6534,28 +6613,28 @@
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="27" t="s">
-        <v>434</v>
+        <v>442</v>
       </c>
       <c r="B1" s="27" t="s">
-        <v>435</v>
+        <v>443</v>
       </c>
       <c r="C1" s="27" t="s">
-        <v>436</v>
+        <v>444</v>
       </c>
       <c r="D1" s="27" t="s">
-        <v>437</v>
+        <v>445</v>
       </c>
       <c r="E1" s="27" t="s">
-        <v>438</v>
+        <v>446</v>
       </c>
       <c r="F1" s="27" t="s">
-        <v>439</v>
+        <v>447</v>
       </c>
       <c r="G1" s="27" t="s">
-        <v>440</v>
+        <v>448</v>
       </c>
       <c r="H1" s="27" t="s">
-        <v>441</v>
+        <v>449</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6585,7 +6664,7 @@
         <v>Add</v>
       </c>
       <c r="H2" s="29" t="s">
-        <v>442</v>
+        <v>450</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6615,7 +6694,7 @@
         <v>OK</v>
       </c>
       <c r="H3" s="29" t="s">
-        <v>443</v>
+        <v>451</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6645,7 +6724,7 @@
         <v>OK</v>
       </c>
       <c r="H4" s="29" t="s">
-        <v>444</v>
+        <v>452</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6675,7 +6754,7 @@
         <v>OK</v>
       </c>
       <c r="H5" s="29" t="s">
-        <v>445</v>
+        <v>453</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6705,7 +6784,7 @@
         <v>OK</v>
       </c>
       <c r="H6" s="29" t="s">
-        <v>446</v>
+        <v>454</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6714,15 +6793,15 @@
       </c>
       <c r="B7" s="29" t="n">
         <f aca="false">COUNTIF(Artifacts!$Q$2:$Q$124,"●")</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C7" s="29" t="n">
         <f aca="false">COUNTIF(Artifacts!$Q$2:$Q$124,"●")+COUNTIF(Artifacts!$Q$2:$Q$124,"○")</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D7" s="29" t="n">
         <f aca="false">COUNTIFS(Artifacts!$Q$2:$Q$124,"●",Artifacts!$R$2:$R$124,"Yes")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E7" s="30" t="n">
         <v>2</v>
@@ -6732,10 +6811,10 @@
       </c>
       <c r="G7" s="29" t="str">
         <f aca="false">IF(D7&lt;E7,"Add",IF(D7&gt;F7,"Trim","OK"))</f>
-        <v>OK</v>
+        <v>Trim</v>
       </c>
       <c r="H7" s="29" t="s">
-        <v>447</v>
+        <v>455</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6750,11 +6829,11 @@
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="28" t="s">
-        <v>448</v>
+        <v>456</v>
       </c>
       <c r="B9" s="29" t="n">
         <f aca="false">COUNTA(Artifacts!$C$2:$C$124)</f>
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C9" s="29"/>
       <c r="D9" s="29"/>
@@ -6765,7 +6844,7 @@
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="31" t="s">
-        <v>449</v>
+        <v>457</v>
       </c>
     </row>
   </sheetData>
@@ -6801,52 +6880,52 @@
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="27" t="s">
-        <v>450</v>
+        <v>458</v>
       </c>
       <c r="B1" s="27" t="s">
-        <v>451</v>
+        <v>459</v>
       </c>
       <c r="C1" s="27" t="s">
-        <v>452</v>
+        <v>460</v>
       </c>
       <c r="D1" s="27" t="s">
-        <v>453</v>
+        <v>461</v>
       </c>
       <c r="E1" s="27" t="s">
-        <v>454</v>
+        <v>462</v>
       </c>
       <c r="F1" s="27" t="s">
-        <v>455</v>
+        <v>463</v>
       </c>
       <c r="G1" s="27" t="s">
-        <v>456</v>
+        <v>464</v>
       </c>
       <c r="H1" s="27" t="s">
-        <v>457</v>
+        <v>465</v>
       </c>
       <c r="I1" s="27" t="s">
-        <v>458</v>
+        <v>466</v>
       </c>
       <c r="J1" s="27" t="s">
-        <v>441</v>
+        <v>449</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="16" t="s">
-        <v>407</v>
+        <v>415</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>459</v>
+        <v>467</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>427</v>
+        <v>435</v>
       </c>
       <c r="D2" s="17"/>
       <c r="E2" s="17" t="s">
         <v>105</v>
       </c>
       <c r="F2" s="17" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="G2" s="17" t="n">
         <v>42.08</v>
@@ -6858,7 +6937,7 @@
         <v>60</v>
       </c>
       <c r="J2" s="21" t="s">
-        <v>460</v>
+        <v>468</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6866,10 +6945,10 @@
         <v>104</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>459</v>
+        <v>467</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>427</v>
+        <v>435</v>
       </c>
       <c r="D3" s="17" t="s">
         <v>105</v>
@@ -6890,7 +6969,7 @@
         <v>60</v>
       </c>
       <c r="J3" s="21" t="s">
-        <v>461</v>
+        <v>469</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6898,10 +6977,10 @@
         <v>87</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>459</v>
+        <v>467</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>419</v>
+        <v>427</v>
       </c>
       <c r="D4" s="17" t="s">
         <v>88</v>
@@ -6910,7 +6989,7 @@
         <v>80</v>
       </c>
       <c r="F4" s="17" t="s">
-        <v>462</v>
+        <v>470</v>
       </c>
       <c r="G4" s="17" t="n">
         <v>41.88</v>
@@ -6922,18 +7001,18 @@
         <v>60</v>
       </c>
       <c r="J4" s="21" t="s">
-        <v>461</v>
+        <v>469</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>463</v>
+        <v>471</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>400</v>
+        <v>408</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>427</v>
+        <v>435</v>
       </c>
       <c r="D5" s="17" t="s">
         <v>80</v>
@@ -6942,7 +7021,7 @@
         <v>70</v>
       </c>
       <c r="F5" s="17" t="s">
-        <v>464</v>
+        <v>472</v>
       </c>
       <c r="G5" s="17" t="n">
         <v>45.46</v>
@@ -6954,7 +7033,7 @@
         <v>60</v>
       </c>
       <c r="J5" s="21" t="s">
-        <v>461</v>
+        <v>469</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6962,10 +7041,10 @@
         <v>69</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>459</v>
+        <v>467</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>427</v>
+        <v>435</v>
       </c>
       <c r="D6" s="17" t="s">
         <v>70</v>
@@ -6974,7 +7053,7 @@
         <v>53</v>
       </c>
       <c r="F6" s="17" t="s">
-        <v>465</v>
+        <v>473</v>
       </c>
       <c r="G6" s="17" t="n">
         <v>32.78</v>
@@ -6986,7 +7065,7 @@
         <v>60</v>
       </c>
       <c r="J6" s="21" t="s">
-        <v>466</v>
+        <v>474</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6994,10 +7073,10 @@
         <v>52</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>459</v>
+        <v>467</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>431</v>
+        <v>439</v>
       </c>
       <c r="D7" s="17" t="s">
         <v>53</v>
@@ -7006,7 +7085,7 @@
         <v>54</v>
       </c>
       <c r="F7" s="17" t="s">
-        <v>467</v>
+        <v>475</v>
       </c>
       <c r="G7" s="17" t="n">
         <v>30.27</v>
@@ -7018,7 +7097,7 @@
         <v>60</v>
       </c>
       <c r="J7" s="21" t="s">
-        <v>468</v>
+        <v>476</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7026,15 +7105,15 @@
         <v>142</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>459</v>
+        <v>467</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>469</v>
+        <v>477</v>
       </c>
       <c r="D8" s="17"/>
       <c r="E8" s="17"/>
       <c r="F8" s="17" t="s">
-        <v>470</v>
+        <v>478</v>
       </c>
       <c r="G8" s="17" t="n">
         <v>29.76</v>
@@ -7052,15 +7131,15 @@
         <v>153</v>
       </c>
       <c r="B9" s="17" t="s">
-        <v>459</v>
+        <v>467</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>469</v>
+        <v>477</v>
       </c>
       <c r="D9" s="17"/>
       <c r="E9" s="17"/>
       <c r="F9" s="17" t="s">
-        <v>471</v>
+        <v>479</v>
       </c>
       <c r="G9" s="17" t="n">
         <v>33.43</v>
@@ -7078,15 +7157,15 @@
         <v>213</v>
       </c>
       <c r="B10" s="17" t="s">
-        <v>459</v>
+        <v>467</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>469</v>
+        <v>477</v>
       </c>
       <c r="D10" s="17"/>
       <c r="E10" s="17"/>
       <c r="F10" s="17" t="s">
-        <v>472</v>
+        <v>480</v>
       </c>
       <c r="G10" s="17" t="n">
         <v>32.76</v>
@@ -7101,13 +7180,13 @@
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="16" t="s">
-        <v>473</v>
+        <v>481</v>
       </c>
       <c r="B11" s="17" t="s">
-        <v>459</v>
+        <v>467</v>
       </c>
       <c r="C11" s="17" t="s">
-        <v>474</v>
+        <v>482</v>
       </c>
       <c r="D11" s="17" t="s">
         <v>88</v>
@@ -7116,7 +7195,7 @@
         <v>88</v>
       </c>
       <c r="F11" s="17" t="s">
-        <v>475</v>
+        <v>483</v>
       </c>
       <c r="G11" s="17" t="n">
         <v>40.81</v>
@@ -7131,22 +7210,22 @@
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="16" t="s">
-        <v>476</v>
+        <v>484</v>
       </c>
       <c r="B12" s="17" t="s">
-        <v>361</v>
+        <v>369</v>
       </c>
       <c r="C12" s="17" t="s">
-        <v>477</v>
+        <v>485</v>
       </c>
       <c r="D12" s="17" t="s">
-        <v>478</v>
+        <v>486</v>
       </c>
       <c r="E12" s="17" t="s">
-        <v>478</v>
+        <v>486</v>
       </c>
       <c r="F12" s="17" t="s">
-        <v>479</v>
+        <v>487</v>
       </c>
       <c r="G12" s="17" t="n">
         <v>39.57</v>
@@ -7161,22 +7240,22 @@
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="16" t="s">
-        <v>480</v>
+        <v>488</v>
       </c>
       <c r="B13" s="17" t="s">
-        <v>370</v>
+        <v>378</v>
       </c>
       <c r="C13" s="17" t="s">
-        <v>477</v>
+        <v>485</v>
       </c>
       <c r="D13" s="17" t="s">
-        <v>478</v>
+        <v>486</v>
       </c>
       <c r="E13" s="17" t="s">
-        <v>478</v>
+        <v>486</v>
       </c>
       <c r="F13" s="17" t="s">
-        <v>481</v>
+        <v>489</v>
       </c>
       <c r="G13" s="17" t="n">
         <v>38.72</v>
@@ -7191,13 +7270,13 @@
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="16" t="s">
-        <v>482</v>
+        <v>490</v>
       </c>
       <c r="B14" s="17" t="s">
-        <v>374</v>
+        <v>382</v>
       </c>
       <c r="C14" s="17" t="s">
-        <v>477</v>
+        <v>485</v>
       </c>
       <c r="D14" s="17" t="s">
         <v>53</v>
@@ -7206,7 +7285,7 @@
         <v>53</v>
       </c>
       <c r="F14" s="17" t="s">
-        <v>483</v>
+        <v>491</v>
       </c>
       <c r="G14" s="17"/>
       <c r="H14" s="17"/>
@@ -7214,18 +7293,18 @@
         <v>60</v>
       </c>
       <c r="J14" s="21" t="s">
-        <v>484</v>
+        <v>492</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="16" t="s">
-        <v>378</v>
+        <v>386</v>
       </c>
       <c r="B15" s="17" t="s">
-        <v>378</v>
+        <v>386</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>477</v>
+        <v>485</v>
       </c>
       <c r="D15" s="17" t="s">
         <v>53</v>
@@ -7234,7 +7313,7 @@
         <v>53</v>
       </c>
       <c r="F15" s="17" t="s">
-        <v>485</v>
+        <v>493</v>
       </c>
       <c r="G15" s="17"/>
       <c r="H15" s="17"/>
@@ -7242,18 +7321,18 @@
         <v>60</v>
       </c>
       <c r="J15" s="21" t="s">
-        <v>484</v>
+        <v>492</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="16" t="s">
-        <v>486</v>
+        <v>494</v>
       </c>
       <c r="B16" s="17" t="s">
-        <v>459</v>
+        <v>467</v>
       </c>
       <c r="C16" s="17" t="s">
-        <v>477</v>
+        <v>485</v>
       </c>
       <c r="D16" s="17" t="s">
         <v>53</v>
@@ -7262,7 +7341,7 @@
         <v>53</v>
       </c>
       <c r="F16" s="17" t="s">
-        <v>487</v>
+        <v>495</v>
       </c>
       <c r="G16" s="17"/>
       <c r="H16" s="17"/>
@@ -7270,18 +7349,18 @@
         <v>60</v>
       </c>
       <c r="J16" s="21" t="s">
-        <v>484</v>
+        <v>492</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="16" t="s">
-        <v>386</v>
+        <v>394</v>
       </c>
       <c r="B17" s="17" t="s">
-        <v>386</v>
+        <v>394</v>
       </c>
       <c r="C17" s="17" t="s">
-        <v>477</v>
+        <v>485</v>
       </c>
       <c r="D17" s="17" t="s">
         <v>71</v>
@@ -7290,7 +7369,7 @@
         <v>71</v>
       </c>
       <c r="F17" s="17" t="s">
-        <v>488</v>
+        <v>496</v>
       </c>
       <c r="G17" s="17" t="n">
         <v>-22.97</v>
@@ -7302,27 +7381,27 @@
         <v>60</v>
       </c>
       <c r="J17" s="21" t="s">
-        <v>489</v>
+        <v>497</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="16" t="s">
-        <v>390</v>
+        <v>398</v>
       </c>
       <c r="B18" s="17" t="s">
-        <v>390</v>
+        <v>398</v>
       </c>
       <c r="C18" s="17" t="s">
-        <v>477</v>
+        <v>485</v>
       </c>
       <c r="D18" s="17" t="s">
-        <v>490</v>
+        <v>498</v>
       </c>
       <c r="E18" s="17" t="s">
-        <v>490</v>
+        <v>498</v>
       </c>
       <c r="F18" s="17" t="s">
-        <v>491</v>
+        <v>499</v>
       </c>
       <c r="G18" s="17"/>
       <c r="H18" s="17"/>
@@ -7330,27 +7409,27 @@
         <v>60</v>
       </c>
       <c r="J18" s="21" t="s">
-        <v>484</v>
+        <v>492</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="16" t="s">
-        <v>492</v>
+        <v>500</v>
       </c>
       <c r="B19" s="17" t="s">
-        <v>459</v>
+        <v>467</v>
       </c>
       <c r="C19" s="17" t="s">
-        <v>477</v>
+        <v>485</v>
       </c>
       <c r="D19" s="17" t="s">
-        <v>490</v>
+        <v>498</v>
       </c>
       <c r="E19" s="17" t="s">
-        <v>490</v>
+        <v>498</v>
       </c>
       <c r="F19" s="17" t="s">
-        <v>493</v>
+        <v>501</v>
       </c>
       <c r="G19" s="17" t="n">
         <v>26.71</v>
@@ -7365,13 +7444,13 @@
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="16" t="s">
-        <v>494</v>
+        <v>502</v>
       </c>
       <c r="B20" s="17" t="s">
-        <v>378</v>
+        <v>386</v>
       </c>
       <c r="C20" s="17" t="s">
-        <v>477</v>
+        <v>485</v>
       </c>
       <c r="D20" s="17" t="s">
         <v>191</v>
@@ -7380,7 +7459,7 @@
         <v>191</v>
       </c>
       <c r="F20" s="17" t="s">
-        <v>495</v>
+        <v>503</v>
       </c>
       <c r="G20" s="17" t="n">
         <v>19.43</v>
@@ -7395,13 +7474,13 @@
     </row>
     <row r="21" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="16" t="s">
-        <v>400</v>
+        <v>408</v>
       </c>
       <c r="B21" s="17" t="s">
-        <v>400</v>
+        <v>408</v>
       </c>
       <c r="C21" s="17" t="s">
-        <v>477</v>
+        <v>485</v>
       </c>
       <c r="D21" s="17" t="s">
         <v>70</v>
@@ -7410,7 +7489,7 @@
         <v>70</v>
       </c>
       <c r="F21" s="17" t="s">
-        <v>496</v>
+        <v>504</v>
       </c>
       <c r="G21" s="17" t="n">
         <v>41.89</v>
@@ -7422,18 +7501,18 @@
         <v>60</v>
       </c>
       <c r="J21" s="21" t="s">
-        <v>497</v>
+        <v>505</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="16" t="s">
-        <v>403</v>
+        <v>411</v>
       </c>
       <c r="B22" s="17" t="s">
-        <v>403</v>
+        <v>411</v>
       </c>
       <c r="C22" s="17" t="s">
-        <v>477</v>
+        <v>485</v>
       </c>
       <c r="D22" s="17" t="s">
         <v>191</v>
@@ -7442,7 +7521,7 @@
         <v>191</v>
       </c>
       <c r="F22" s="17" t="s">
-        <v>498</v>
+        <v>506</v>
       </c>
       <c r="G22" s="17"/>
       <c r="H22" s="17"/>
@@ -7453,12 +7532,12 @@
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="31" t="s">
-        <v>499</v>
+        <v>507</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="31" t="s">
-        <v>500</v>
+        <v>508</v>
       </c>
     </row>
   </sheetData>
@@ -7494,33 +7573,33 @@
         <v>24</v>
       </c>
       <c r="B1" s="27" t="s">
-        <v>501</v>
+        <v>509</v>
       </c>
       <c r="C1" s="27" t="s">
-        <v>450</v>
+        <v>458</v>
       </c>
       <c r="D1" s="27" t="s">
-        <v>502</v>
+        <v>510</v>
       </c>
       <c r="E1" s="27" t="s">
-        <v>367</v>
+        <v>375</v>
       </c>
       <c r="F1" s="27" t="s">
         <v>41</v>
       </c>
       <c r="G1" s="27" t="s">
-        <v>441</v>
+        <v>449</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="32" t="s">
-        <v>357</v>
+        <v>365</v>
       </c>
       <c r="B2" s="33" t="s">
-        <v>358</v>
+        <v>366</v>
       </c>
       <c r="C2" s="32" t="s">
-        <v>361</v>
+        <v>369</v>
       </c>
       <c r="D2" s="32" t="n">
         <v>2026</v>
@@ -7535,13 +7614,13 @@
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="32" t="s">
-        <v>368</v>
+        <v>376</v>
       </c>
       <c r="B3" s="33" t="s">
-        <v>369</v>
+        <v>377</v>
       </c>
       <c r="C3" s="32" t="s">
-        <v>370</v>
+        <v>378</v>
       </c>
       <c r="D3" s="32" t="n">
         <v>2026</v>
@@ -7556,13 +7635,13 @@
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="32" t="s">
-        <v>372</v>
+        <v>380</v>
       </c>
       <c r="B4" s="33" t="s">
-        <v>373</v>
+        <v>381</v>
       </c>
       <c r="C4" s="32" t="s">
-        <v>374</v>
+        <v>382</v>
       </c>
       <c r="D4" s="32" t="s">
         <v>53</v>
@@ -7577,13 +7656,13 @@
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="32" t="s">
-        <v>376</v>
+        <v>384</v>
       </c>
       <c r="B5" s="33" t="s">
-        <v>377</v>
+        <v>385</v>
       </c>
       <c r="C5" s="32" t="s">
-        <v>378</v>
+        <v>386</v>
       </c>
       <c r="D5" s="32" t="s">
         <v>53</v>
@@ -7598,13 +7677,13 @@
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="32" t="s">
-        <v>380</v>
+        <v>388</v>
       </c>
       <c r="B6" s="33" t="s">
-        <v>381</v>
+        <v>389</v>
       </c>
       <c r="C6" s="32" t="s">
-        <v>382</v>
+        <v>390</v>
       </c>
       <c r="D6" s="32" t="s">
         <v>53</v>
@@ -7619,13 +7698,13 @@
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="32" t="s">
-        <v>384</v>
+        <v>392</v>
       </c>
       <c r="B7" s="33" t="s">
-        <v>385</v>
+        <v>393</v>
       </c>
       <c r="C7" s="32" t="s">
-        <v>386</v>
+        <v>394</v>
       </c>
       <c r="D7" s="32" t="n">
         <v>2024</v>
@@ -7640,13 +7719,13 @@
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="32" t="s">
-        <v>388</v>
+        <v>396</v>
       </c>
       <c r="B8" s="33" t="s">
-        <v>389</v>
+        <v>397</v>
       </c>
       <c r="C8" s="32" t="s">
-        <v>390</v>
+        <v>398</v>
       </c>
       <c r="D8" s="32" t="n">
         <v>2023</v>
@@ -7661,13 +7740,13 @@
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="32" t="s">
-        <v>392</v>
+        <v>400</v>
       </c>
       <c r="B9" s="33" t="s">
-        <v>393</v>
+        <v>401</v>
       </c>
       <c r="C9" s="32" t="s">
-        <v>394</v>
+        <v>402</v>
       </c>
       <c r="D9" s="32" t="n">
         <v>2023</v>
@@ -7682,13 +7761,13 @@
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="32" t="s">
-        <v>395</v>
+        <v>403</v>
       </c>
       <c r="B10" s="33" t="s">
-        <v>396</v>
+        <v>404</v>
       </c>
       <c r="C10" s="32" t="s">
-        <v>378</v>
+        <v>386</v>
       </c>
       <c r="D10" s="32" t="n">
         <v>2022</v>
@@ -7703,13 +7782,13 @@
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="32" t="s">
-        <v>398</v>
+        <v>406</v>
       </c>
       <c r="B11" s="33" t="s">
-        <v>399</v>
+        <v>407</v>
       </c>
       <c r="C11" s="32" t="s">
-        <v>400</v>
+        <v>408</v>
       </c>
       <c r="D11" s="32" t="n">
         <v>2021</v>
@@ -7724,13 +7803,13 @@
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="32" t="s">
-        <v>401</v>
+        <v>409</v>
       </c>
       <c r="B12" s="33" t="s">
-        <v>402</v>
+        <v>410</v>
       </c>
       <c r="C12" s="32" t="s">
-        <v>403</v>
+        <v>411</v>
       </c>
       <c r="D12" s="32" t="n">
         <v>2022</v>
@@ -7745,7 +7824,7 @@
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="D13" s="28" t="s">
-        <v>503</v>
+        <v>511</v>
       </c>
       <c r="E13" s="28" t="n">
         <f aca="false">SUM(E2:E12)</f>
@@ -7754,7 +7833,7 @@
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="D14" s="28" t="s">
-        <v>504</v>
+        <v>512</v>
       </c>
       <c r="E14" s="28" t="n">
         <f aca="false">COUNTIF(F2:F12,"Yes")</f>
@@ -7763,12 +7842,12 @@
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="31" t="s">
-        <v>505</v>
+        <v>513</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>506</v>
+        <v>514</v>
       </c>
     </row>
   </sheetData>
@@ -7798,19 +7877,19 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="27" t="s">
-        <v>507</v>
+        <v>515</v>
       </c>
       <c r="B1" s="27" t="s">
-        <v>451</v>
+        <v>459</v>
       </c>
       <c r="C1" s="27" t="s">
-        <v>508</v>
+        <v>516</v>
       </c>
       <c r="D1" s="27" t="s">
-        <v>509</v>
+        <v>517</v>
       </c>
       <c r="E1" s="27" t="s">
-        <v>441</v>
+        <v>449</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7818,13 +7897,13 @@
         <v>1</v>
       </c>
       <c r="B2" s="33" t="s">
-        <v>459</v>
+        <v>467</v>
       </c>
       <c r="C2" s="33" t="s">
-        <v>510</v>
+        <v>518</v>
       </c>
       <c r="D2" s="33" t="s">
-        <v>511</v>
+        <v>519</v>
       </c>
       <c r="E2" s="33"/>
     </row>
@@ -7833,13 +7912,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="33" t="s">
-        <v>512</v>
+        <v>520</v>
       </c>
       <c r="C3" s="33" t="s">
-        <v>510</v>
+        <v>518</v>
       </c>
       <c r="D3" s="33" t="s">
-        <v>511</v>
+        <v>519</v>
       </c>
       <c r="E3" s="33"/>
     </row>
@@ -7848,13 +7927,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="33" t="s">
-        <v>378</v>
+        <v>386</v>
       </c>
       <c r="C4" s="33" t="s">
-        <v>510</v>
+        <v>518</v>
       </c>
       <c r="D4" s="33" t="s">
-        <v>511</v>
+        <v>519</v>
       </c>
       <c r="E4" s="33"/>
     </row>
@@ -7863,13 +7942,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="33" t="s">
-        <v>513</v>
+        <v>521</v>
       </c>
       <c r="C5" s="33" t="s">
-        <v>514</v>
+        <v>522</v>
       </c>
       <c r="D5" s="33" t="s">
-        <v>511</v>
+        <v>519</v>
       </c>
       <c r="E5" s="33"/>
     </row>
@@ -7878,13 +7957,13 @@
         <v>5</v>
       </c>
       <c r="B6" s="33" t="s">
-        <v>515</v>
+        <v>523</v>
       </c>
       <c r="C6" s="33" t="s">
-        <v>514</v>
+        <v>522</v>
       </c>
       <c r="D6" s="33" t="s">
-        <v>511</v>
+        <v>519</v>
       </c>
       <c r="E6" s="33"/>
     </row>
@@ -7893,16 +7972,16 @@
         <v>6</v>
       </c>
       <c r="B7" s="33" t="s">
-        <v>516</v>
+        <v>524</v>
       </c>
       <c r="C7" s="33" t="s">
-        <v>514</v>
+        <v>522</v>
       </c>
       <c r="D7" s="33" t="s">
-        <v>517</v>
+        <v>525</v>
       </c>
       <c r="E7" s="33" t="s">
-        <v>518</v>
+        <v>526</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7910,16 +7989,16 @@
         <v>7</v>
       </c>
       <c r="B8" s="33" t="s">
-        <v>519</v>
+        <v>527</v>
       </c>
       <c r="C8" s="33" t="s">
-        <v>514</v>
+        <v>522</v>
       </c>
       <c r="D8" s="33" t="s">
-        <v>517</v>
+        <v>525</v>
       </c>
       <c r="E8" s="33" t="s">
-        <v>518</v>
+        <v>526</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7927,16 +8006,16 @@
         <v>8</v>
       </c>
       <c r="B9" s="33" t="s">
-        <v>520</v>
+        <v>528</v>
       </c>
       <c r="C9" s="33" t="s">
-        <v>514</v>
+        <v>522</v>
       </c>
       <c r="D9" s="33" t="s">
-        <v>517</v>
+        <v>525</v>
       </c>
       <c r="E9" s="33" t="s">
-        <v>518</v>
+        <v>526</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7944,16 +8023,16 @@
         <v>9</v>
       </c>
       <c r="B10" s="33" t="s">
-        <v>521</v>
+        <v>529</v>
       </c>
       <c r="C10" s="33" t="s">
-        <v>514</v>
+        <v>522</v>
       </c>
       <c r="D10" s="33" t="s">
-        <v>517</v>
+        <v>525</v>
       </c>
       <c r="E10" s="33" t="s">
-        <v>518</v>
+        <v>526</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7961,13 +8040,13 @@
         <v>10</v>
       </c>
       <c r="B11" s="33" t="s">
+        <v>530</v>
+      </c>
+      <c r="C11" s="33" t="s">
         <v>522</v>
       </c>
-      <c r="C11" s="33" t="s">
-        <v>514</v>
-      </c>
       <c r="D11" s="33" t="s">
-        <v>511</v>
+        <v>519</v>
       </c>
       <c r="E11" s="33"/>
     </row>
@@ -7976,13 +8055,13 @@
         <v>11</v>
       </c>
       <c r="B12" s="33" t="s">
-        <v>523</v>
+        <v>531</v>
       </c>
       <c r="C12" s="33" t="s">
-        <v>524</v>
+        <v>532</v>
       </c>
       <c r="D12" s="33" t="s">
-        <v>511</v>
+        <v>519</v>
       </c>
       <c r="E12" s="33"/>
     </row>
@@ -7991,13 +8070,13 @@
         <v>12</v>
       </c>
       <c r="B13" s="33" t="s">
-        <v>525</v>
+        <v>533</v>
       </c>
       <c r="C13" s="33" t="s">
-        <v>524</v>
+        <v>532</v>
       </c>
       <c r="D13" s="33" t="s">
-        <v>511</v>
+        <v>519</v>
       </c>
       <c r="E13" s="33"/>
     </row>
@@ -8006,13 +8085,13 @@
         <v>13</v>
       </c>
       <c r="B14" s="33" t="s">
-        <v>526</v>
+        <v>534</v>
       </c>
       <c r="C14" s="33" t="s">
-        <v>524</v>
+        <v>532</v>
       </c>
       <c r="D14" s="33" t="s">
-        <v>511</v>
+        <v>519</v>
       </c>
       <c r="E14" s="33"/>
     </row>
@@ -8021,13 +8100,13 @@
         <v>14</v>
       </c>
       <c r="B15" s="33" t="s">
-        <v>527</v>
+        <v>535</v>
       </c>
       <c r="C15" s="33" t="s">
-        <v>524</v>
+        <v>532</v>
       </c>
       <c r="D15" s="33" t="s">
-        <v>511</v>
+        <v>519</v>
       </c>
       <c r="E15" s="33"/>
     </row>
@@ -8036,16 +8115,16 @@
         <v>15</v>
       </c>
       <c r="B16" s="33" t="s">
-        <v>403</v>
+        <v>411</v>
       </c>
       <c r="C16" s="33" t="s">
-        <v>528</v>
+        <v>536</v>
       </c>
       <c r="D16" s="33" t="s">
-        <v>511</v>
+        <v>519</v>
       </c>
       <c r="E16" s="33" t="s">
-        <v>498</v>
+        <v>506</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8053,16 +8132,16 @@
         <v>16</v>
       </c>
       <c r="B17" s="33" t="s">
-        <v>390</v>
+        <v>398</v>
       </c>
       <c r="C17" s="33" t="s">
-        <v>528</v>
+        <v>536</v>
       </c>
       <c r="D17" s="33" t="s">
-        <v>511</v>
+        <v>519</v>
       </c>
       <c r="E17" s="33" t="s">
-        <v>529</v>
+        <v>537</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8070,16 +8149,16 @@
         <v>17</v>
       </c>
       <c r="B18" s="33" t="s">
-        <v>386</v>
+        <v>394</v>
       </c>
       <c r="C18" s="33" t="s">
-        <v>528</v>
+        <v>536</v>
       </c>
       <c r="D18" s="33" t="s">
-        <v>511</v>
+        <v>519</v>
       </c>
       <c r="E18" s="33" t="s">
-        <v>488</v>
+        <v>496</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8087,16 +8166,16 @@
         <v>18</v>
       </c>
       <c r="B19" s="33" t="s">
-        <v>530</v>
+        <v>538</v>
       </c>
       <c r="C19" s="33" t="s">
-        <v>528</v>
+        <v>536</v>
       </c>
       <c r="D19" s="33" t="s">
-        <v>511</v>
+        <v>519</v>
       </c>
       <c r="E19" s="33" t="s">
-        <v>483</v>
+        <v>491</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8104,16 +8183,16 @@
         <v>19</v>
       </c>
       <c r="B20" s="33" t="s">
-        <v>531</v>
+        <v>539</v>
       </c>
       <c r="C20" s="33" t="s">
-        <v>528</v>
+        <v>536</v>
       </c>
       <c r="D20" s="33" t="s">
-        <v>511</v>
+        <v>519</v>
       </c>
       <c r="E20" s="33" t="s">
-        <v>483</v>
+        <v>491</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8121,13 +8200,13 @@
         <v>20</v>
       </c>
       <c r="B21" s="33" t="s">
-        <v>532</v>
+        <v>540</v>
       </c>
       <c r="C21" s="33" t="s">
-        <v>533</v>
+        <v>541</v>
       </c>
       <c r="D21" s="33" t="s">
-        <v>511</v>
+        <v>519</v>
       </c>
       <c r="E21" s="33"/>
     </row>
@@ -8136,16 +8215,16 @@
         <v>21</v>
       </c>
       <c r="B22" s="33" t="s">
-        <v>361</v>
+        <v>369</v>
       </c>
       <c r="C22" s="33" t="s">
-        <v>534</v>
+        <v>542</v>
       </c>
       <c r="D22" s="33" t="s">
-        <v>511</v>
+        <v>519</v>
       </c>
       <c r="E22" s="33" t="s">
-        <v>479</v>
+        <v>487</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8153,16 +8232,16 @@
         <v>22</v>
       </c>
       <c r="B23" s="33" t="s">
-        <v>370</v>
+        <v>378</v>
       </c>
       <c r="C23" s="33" t="s">
-        <v>534</v>
+        <v>542</v>
       </c>
       <c r="D23" s="33" t="s">
-        <v>511</v>
+        <v>519</v>
       </c>
       <c r="E23" s="33" t="s">
-        <v>481</v>
+        <v>489</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8170,16 +8249,16 @@
         <v>23</v>
       </c>
       <c r="B24" s="33" t="s">
-        <v>400</v>
+        <v>408</v>
       </c>
       <c r="C24" s="33" t="s">
-        <v>534</v>
+        <v>542</v>
       </c>
       <c r="D24" s="33" t="s">
-        <v>511</v>
+        <v>519</v>
       </c>
       <c r="E24" s="33" t="s">
-        <v>535</v>
+        <v>543</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8187,13 +8266,13 @@
         <v>24</v>
       </c>
       <c r="B25" s="33" t="s">
-        <v>536</v>
+        <v>544</v>
       </c>
       <c r="C25" s="33" t="s">
-        <v>534</v>
+        <v>542</v>
       </c>
       <c r="D25" s="33" t="s">
-        <v>511</v>
+        <v>519</v>
       </c>
       <c r="E25" s="33"/>
     </row>
@@ -8202,13 +8281,13 @@
         <v>25</v>
       </c>
       <c r="B26" s="33" t="s">
-        <v>537</v>
+        <v>545</v>
       </c>
       <c r="C26" s="33" t="s">
-        <v>534</v>
+        <v>542</v>
       </c>
       <c r="D26" s="33" t="s">
-        <v>511</v>
+        <v>519</v>
       </c>
       <c r="E26" s="33"/>
     </row>
@@ -8217,13 +8296,13 @@
         <v>26</v>
       </c>
       <c r="B27" s="33" t="s">
-        <v>538</v>
+        <v>546</v>
       </c>
       <c r="C27" s="33" t="s">
-        <v>534</v>
+        <v>542</v>
       </c>
       <c r="D27" s="33" t="s">
-        <v>511</v>
+        <v>519</v>
       </c>
       <c r="E27" s="33"/>
     </row>
@@ -8232,13 +8311,13 @@
         <v>27</v>
       </c>
       <c r="B28" s="33" t="s">
-        <v>539</v>
+        <v>547</v>
       </c>
       <c r="C28" s="33" t="s">
-        <v>534</v>
+        <v>542</v>
       </c>
       <c r="D28" s="33" t="s">
-        <v>511</v>
+        <v>519</v>
       </c>
       <c r="E28" s="33"/>
     </row>
@@ -8247,13 +8326,13 @@
         <v>28</v>
       </c>
       <c r="B29" s="33" t="s">
-        <v>540</v>
+        <v>548</v>
       </c>
       <c r="C29" s="33" t="s">
-        <v>534</v>
+        <v>542</v>
       </c>
       <c r="D29" s="33" t="s">
-        <v>511</v>
+        <v>519</v>
       </c>
       <c r="E29" s="33"/>
     </row>
@@ -8262,13 +8341,13 @@
         <v>29</v>
       </c>
       <c r="B30" s="33" t="s">
-        <v>541</v>
+        <v>549</v>
       </c>
       <c r="C30" s="33" t="s">
-        <v>534</v>
+        <v>542</v>
       </c>
       <c r="D30" s="33" t="s">
-        <v>511</v>
+        <v>519</v>
       </c>
       <c r="E30" s="33"/>
     </row>
@@ -8277,13 +8356,13 @@
         <v>30</v>
       </c>
       <c r="B31" s="33" t="s">
+        <v>550</v>
+      </c>
+      <c r="C31" s="33" t="s">
         <v>542</v>
       </c>
-      <c r="C31" s="33" t="s">
-        <v>534</v>
-      </c>
       <c r="D31" s="33" t="s">
-        <v>511</v>
+        <v>519</v>
       </c>
       <c r="E31" s="33"/>
     </row>
@@ -8292,13 +8371,13 @@
         <v>31</v>
       </c>
       <c r="B32" s="33" t="s">
-        <v>543</v>
+        <v>551</v>
       </c>
       <c r="C32" s="33" t="s">
-        <v>534</v>
+        <v>542</v>
       </c>
       <c r="D32" s="33" t="s">
-        <v>511</v>
+        <v>519</v>
       </c>
       <c r="E32" s="33"/>
     </row>
@@ -8307,13 +8386,13 @@
         <v>32</v>
       </c>
       <c r="B33" s="33" t="s">
-        <v>544</v>
+        <v>552</v>
       </c>
       <c r="C33" s="33" t="s">
-        <v>534</v>
+        <v>542</v>
       </c>
       <c r="D33" s="33" t="s">
-        <v>511</v>
+        <v>519</v>
       </c>
       <c r="E33" s="33"/>
     </row>
@@ -8322,13 +8401,13 @@
         <v>33</v>
       </c>
       <c r="B34" s="33" t="s">
-        <v>545</v>
+        <v>553</v>
       </c>
       <c r="C34" s="33" t="s">
-        <v>534</v>
+        <v>542</v>
       </c>
       <c r="D34" s="33" t="s">
-        <v>511</v>
+        <v>519</v>
       </c>
       <c r="E34" s="33"/>
     </row>
@@ -8337,19 +8416,19 @@
         <v>34</v>
       </c>
       <c r="B35" s="33" t="s">
-        <v>546</v>
+        <v>554</v>
       </c>
       <c r="C35" s="33" t="s">
-        <v>534</v>
+        <v>542</v>
       </c>
       <c r="D35" s="33" t="s">
-        <v>511</v>
+        <v>519</v>
       </c>
       <c r="E35" s="33"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B37" s="28" t="s">
-        <v>503</v>
+        <v>511</v>
       </c>
       <c r="C37" s="28" t="n">
         <f aca="false">COUNTA(B2:B35)</f>
@@ -8358,7 +8437,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="1" t="s">
-        <v>511</v>
+        <v>519</v>
       </c>
       <c r="C38" s="1" t="n">
         <f aca="false">COUNTIF(D2:D35,"Shaded")</f>
@@ -8367,7 +8446,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B39" s="1" t="s">
-        <v>517</v>
+        <v>525</v>
       </c>
       <c r="C39" s="1" t="n">
         <f aca="false">COUNTIF(D2:D35,"Dot")</f>
@@ -8376,7 +8455,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="31" t="s">
-        <v>547</v>
+        <v>555</v>
       </c>
     </row>
   </sheetData>
@@ -8407,16 +8486,16 @@
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="27" t="s">
-        <v>548</v>
+        <v>556</v>
       </c>
       <c r="B1" s="27" t="s">
-        <v>549</v>
+        <v>557</v>
       </c>
       <c r="C1" s="27" t="s">
-        <v>550</v>
+        <v>558</v>
       </c>
       <c r="D1" s="27" t="s">
-        <v>551</v>
+        <v>559</v>
       </c>
       <c r="E1" s="27" t="s">
         <v>46</v>
@@ -8424,98 +8503,98 @@
     </row>
     <row r="2" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="17" t="s">
-        <v>552</v>
+        <v>560</v>
       </c>
       <c r="B2" s="16" t="s">
-        <v>553</v>
+        <v>561</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>554</v>
+        <v>562</v>
       </c>
       <c r="D2" s="21" t="s">
         <v>60</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>555</v>
+        <v>563</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="17" t="s">
-        <v>552</v>
+        <v>560</v>
       </c>
       <c r="B3" s="16" t="s">
-        <v>556</v>
+        <v>564</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>557</v>
+        <v>565</v>
       </c>
       <c r="D3" s="21" t="s">
         <v>60</v>
       </c>
       <c r="E3" s="17" t="s">
-        <v>555</v>
+        <v>563</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="17" t="s">
-        <v>552</v>
+        <v>560</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>558</v>
+        <v>566</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>559</v>
+        <v>567</v>
       </c>
       <c r="D4" s="21" t="s">
         <v>60</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>555</v>
+        <v>563</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="17" t="s">
-        <v>552</v>
+        <v>560</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>560</v>
+        <v>568</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>561</v>
+        <v>569</v>
       </c>
       <c r="D5" s="21" t="s">
         <v>60</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>555</v>
+        <v>563</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="17" t="s">
-        <v>552</v>
+        <v>560</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>562</v>
+        <v>570</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>563</v>
+        <v>571</v>
       </c>
       <c r="D6" s="21" t="s">
         <v>60</v>
       </c>
       <c r="E6" s="17" t="s">
-        <v>555</v>
+        <v>563</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="17" t="s">
-        <v>564</v>
+        <v>572</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>565</v>
+        <v>573</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>566</v>
+        <v>574</v>
       </c>
       <c r="D7" s="21" t="s">
         <v>60</v>
@@ -8526,13 +8605,13 @@
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="17" t="s">
-        <v>564</v>
+        <v>572</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>567</v>
+        <v>575</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>568</v>
+        <v>576</v>
       </c>
       <c r="D8" s="21" t="s">
         <v>60</v>
@@ -8543,19 +8622,19 @@
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="17" t="s">
-        <v>564</v>
+        <v>572</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>569</v>
+        <v>577</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>570</v>
+        <v>578</v>
       </c>
       <c r="D9" s="21" t="s">
         <v>60</v>
       </c>
       <c r="E9" s="17" t="s">
-        <v>555</v>
+        <v>563</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8563,110 +8642,110 @@
         <v>247</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>571</v>
+        <v>579</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>572</v>
+        <v>580</v>
       </c>
       <c r="D10" s="21" t="s">
         <v>60</v>
       </c>
       <c r="E10" s="17" t="s">
-        <v>555</v>
+        <v>563</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="17" t="s">
-        <v>573</v>
+        <v>581</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>574</v>
+        <v>582</v>
       </c>
       <c r="C11" s="17"/>
       <c r="D11" s="21" t="s">
         <v>60</v>
       </c>
       <c r="E11" s="17" t="s">
-        <v>555</v>
+        <v>563</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="17" t="s">
-        <v>573</v>
+        <v>581</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>575</v>
+        <v>583</v>
       </c>
       <c r="C12" s="17" t="s">
-        <v>576</v>
+        <v>584</v>
       </c>
       <c r="D12" s="21" t="s">
         <v>60</v>
       </c>
       <c r="E12" s="17" t="s">
-        <v>555</v>
+        <v>563</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="17" t="s">
-        <v>573</v>
+        <v>581</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>577</v>
+        <v>585</v>
       </c>
       <c r="C13" s="17" t="s">
-        <v>578</v>
+        <v>586</v>
       </c>
       <c r="D13" s="21" t="s">
         <v>60</v>
       </c>
       <c r="E13" s="17" t="s">
-        <v>555</v>
+        <v>563</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="17" t="s">
-        <v>573</v>
+        <v>581</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>579</v>
+        <v>587</v>
       </c>
       <c r="C14" s="17" t="s">
-        <v>580</v>
+        <v>588</v>
       </c>
       <c r="D14" s="21" t="s">
         <v>60</v>
       </c>
       <c r="E14" s="17" t="s">
-        <v>555</v>
+        <v>563</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="17" t="s">
-        <v>581</v>
+        <v>589</v>
       </c>
       <c r="B15" s="16" t="s">
-        <v>581</v>
+        <v>589</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>582</v>
+        <v>590</v>
       </c>
       <c r="D15" s="21" t="s">
         <v>60</v>
       </c>
       <c r="E15" s="17" t="s">
-        <v>555</v>
+        <v>563</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="17" t="s">
-        <v>583</v>
+        <v>591</v>
       </c>
       <c r="B16" s="16" t="s">
-        <v>583</v>
+        <v>591</v>
       </c>
       <c r="C16" s="17" t="s">
-        <v>584</v>
+        <v>592</v>
       </c>
       <c r="D16" s="21" t="s">
         <v>60</v>
@@ -8677,13 +8756,13 @@
     </row>
     <row r="17" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="17" t="s">
-        <v>585</v>
+        <v>593</v>
       </c>
       <c r="B17" s="16" t="s">
-        <v>586</v>
+        <v>594</v>
       </c>
       <c r="C17" s="17" t="s">
-        <v>587</v>
+        <v>595</v>
       </c>
       <c r="D17" s="21" t="s">
         <v>60</v>
@@ -8694,13 +8773,13 @@
     </row>
     <row r="18" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="17" t="s">
-        <v>585</v>
+        <v>593</v>
       </c>
       <c r="B18" s="16" t="s">
-        <v>588</v>
+        <v>596</v>
       </c>
       <c r="C18" s="17" t="s">
-        <v>589</v>
+        <v>597</v>
       </c>
       <c r="D18" s="21" t="s">
         <v>60</v>
@@ -8711,13 +8790,13 @@
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="17" t="s">
-        <v>585</v>
+        <v>593</v>
       </c>
       <c r="B19" s="16" t="s">
-        <v>590</v>
+        <v>598</v>
       </c>
       <c r="C19" s="17" t="s">
-        <v>591</v>
+        <v>599</v>
       </c>
       <c r="D19" s="21" t="s">
         <v>60</v>
@@ -8728,13 +8807,13 @@
     </row>
     <row r="20" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="17" t="s">
-        <v>585</v>
+        <v>593</v>
       </c>
       <c r="B20" s="16" t="s">
-        <v>592</v>
+        <v>600</v>
       </c>
       <c r="C20" s="17" t="s">
-        <v>593</v>
+        <v>601</v>
       </c>
       <c r="D20" s="21" t="s">
         <v>60</v>
@@ -8745,64 +8824,64 @@
     </row>
     <row r="21" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="17" t="s">
-        <v>594</v>
+        <v>602</v>
       </c>
       <c r="B21" s="16" t="s">
-        <v>595</v>
+        <v>603</v>
       </c>
       <c r="C21" s="17" t="s">
-        <v>596</v>
+        <v>604</v>
       </c>
       <c r="D21" s="21" t="s">
-        <v>597</v>
+        <v>605</v>
       </c>
       <c r="E21" s="17" t="s">
-        <v>598</v>
+        <v>606</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="17" t="s">
-        <v>599</v>
+        <v>607</v>
       </c>
       <c r="B22" s="16" t="s">
-        <v>600</v>
+        <v>608</v>
       </c>
       <c r="C22" s="17" t="s">
-        <v>601</v>
+        <v>609</v>
       </c>
       <c r="D22" s="21"/>
       <c r="E22" s="17" t="s">
-        <v>555</v>
+        <v>563</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="17" t="s">
-        <v>599</v>
+        <v>607</v>
       </c>
       <c r="B23" s="16" t="s">
-        <v>602</v>
+        <v>610</v>
       </c>
       <c r="C23" s="17" t="s">
-        <v>603</v>
+        <v>611</v>
       </c>
       <c r="D23" s="21"/>
       <c r="E23" s="17" t="s">
-        <v>555</v>
+        <v>563</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="17" t="s">
-        <v>599</v>
+        <v>607</v>
       </c>
       <c r="B24" s="16" t="s">
-        <v>604</v>
+        <v>612</v>
       </c>
       <c r="C24" s="17" t="s">
-        <v>605</v>
+        <v>613</v>
       </c>
       <c r="D24" s="21"/>
       <c r="E24" s="17" t="s">
-        <v>606</v>
+        <v>614</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="99.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8810,24 +8889,24 @@
         <v>247</v>
       </c>
       <c r="B25" s="16" t="s">
-        <v>607</v>
+        <v>615</v>
       </c>
       <c r="C25" s="17" t="s">
-        <v>608</v>
+        <v>616</v>
       </c>
       <c r="D25" s="21" t="s">
         <v>60</v>
       </c>
       <c r="E25" s="17" t="s">
-        <v>606</v>
+        <v>614</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
-        <v>609</v>
+        <v>617</v>
       </c>
       <c r="B26" s="29" t="s">
-        <v>610</v>
+        <v>618</v>
       </c>
     </row>
   </sheetData>
@@ -8846,7 +8925,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4"/>
@@ -8857,16 +8936,16 @@
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="27" t="s">
-        <v>507</v>
+        <v>515</v>
       </c>
       <c r="B1" s="27" t="s">
-        <v>611</v>
+        <v>619</v>
       </c>
       <c r="C1" s="27" t="s">
-        <v>612</v>
+        <v>620</v>
       </c>
       <c r="D1" s="27" t="s">
-        <v>606</v>
+        <v>614</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8874,10 +8953,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>613</v>
+        <v>621</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>614</v>
+        <v>622</v>
       </c>
       <c r="D2" s="21" t="s">
         <v>60</v>
@@ -8888,13 +8967,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>615</v>
+        <v>623</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>616</v>
+        <v>624</v>
       </c>
       <c r="D3" s="21" t="s">
-        <v>617</v>
+        <v>625</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8902,13 +8981,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>618</v>
+        <v>626</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>619</v>
+        <v>627</v>
       </c>
       <c r="D4" s="21" t="s">
-        <v>620</v>
+        <v>628</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8916,13 +8995,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>621</v>
+        <v>629</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>622</v>
+        <v>630</v>
       </c>
       <c r="D5" s="21" t="s">
-        <v>623</v>
+        <v>631</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8930,13 +9009,13 @@
         <v>5</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>624</v>
+        <v>632</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>625</v>
+        <v>633</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>626</v>
+        <v>634</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8944,13 +9023,13 @@
         <v>6</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>627</v>
+        <v>635</v>
       </c>
       <c r="C7" s="17" t="s">
         <v>206</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>628</v>
+        <v>636</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8958,13 +9037,13 @@
         <v>7</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>629</v>
+        <v>637</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>630</v>
+        <v>638</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>631</v>
+        <v>639</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8972,13 +9051,13 @@
         <v>8</v>
       </c>
       <c r="B9" s="17" t="s">
-        <v>632</v>
+        <v>640</v>
       </c>
       <c r="C9" s="17" t="s">
         <v>177</v>
       </c>
       <c r="D9" s="21" t="s">
-        <v>633</v>
+        <v>641</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8986,13 +9065,13 @@
         <v>9</v>
       </c>
       <c r="B10" s="17" t="s">
-        <v>634</v>
+        <v>642</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>635</v>
+        <v>643</v>
       </c>
       <c r="D10" s="21" t="s">
-        <v>636</v>
+        <v>644</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9000,13 +9079,13 @@
         <v>10</v>
       </c>
       <c r="B11" s="17" t="s">
-        <v>637</v>
+        <v>645</v>
       </c>
       <c r="C11" s="17" t="s">
-        <v>638</v>
+        <v>646</v>
       </c>
       <c r="D11" s="21" t="s">
-        <v>639</v>
+        <v>647</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9014,13 +9093,13 @@
         <v>11</v>
       </c>
       <c r="B12" s="17" t="s">
-        <v>640</v>
+        <v>648</v>
       </c>
       <c r="C12" s="17" t="s">
         <v>233</v>
       </c>
       <c r="D12" s="21" t="s">
-        <v>641</v>
+        <v>649</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9028,13 +9107,13 @@
         <v>12</v>
       </c>
       <c r="B13" s="17" t="s">
-        <v>642</v>
+        <v>650</v>
       </c>
       <c r="C13" s="17" t="s">
-        <v>643</v>
+        <v>651</v>
       </c>
       <c r="D13" s="21" t="s">
-        <v>644</v>
+        <v>652</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9042,13 +9121,13 @@
         <v>13</v>
       </c>
       <c r="B14" s="17" t="s">
-        <v>645</v>
+        <v>653</v>
       </c>
       <c r="C14" s="17" t="s">
-        <v>646</v>
+        <v>654</v>
       </c>
       <c r="D14" s="21" t="s">
-        <v>647</v>
+        <v>655</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9056,13 +9135,13 @@
         <v>14</v>
       </c>
       <c r="B15" s="17" t="s">
-        <v>648</v>
+        <v>656</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>649</v>
+        <v>657</v>
       </c>
       <c r="D15" s="21" t="s">
-        <v>650</v>
+        <v>658</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9070,13 +9149,13 @@
         <v>15</v>
       </c>
       <c r="B16" s="17" t="s">
-        <v>651</v>
+        <v>659</v>
       </c>
       <c r="C16" s="17" t="s">
-        <v>652</v>
+        <v>660</v>
       </c>
       <c r="D16" s="21" t="s">
-        <v>653</v>
+        <v>661</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9084,13 +9163,13 @@
         <v>16</v>
       </c>
       <c r="B17" s="17" t="s">
-        <v>654</v>
+        <v>662</v>
       </c>
       <c r="C17" s="17" t="s">
         <v>35</v>
       </c>
       <c r="D17" s="21" t="s">
-        <v>655</v>
+        <v>663</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9098,13 +9177,13 @@
         <v>17</v>
       </c>
       <c r="B18" s="17" t="s">
-        <v>656</v>
+        <v>664</v>
       </c>
       <c r="C18" s="17" t="s">
         <v>35</v>
       </c>
       <c r="D18" s="21" t="s">
-        <v>657</v>
+        <v>665</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9112,13 +9191,13 @@
         <v>18</v>
       </c>
       <c r="B19" s="17" t="s">
-        <v>658</v>
+        <v>666</v>
       </c>
       <c r="C19" s="17" t="s">
-        <v>659</v>
+        <v>667</v>
       </c>
       <c r="D19" s="21" t="s">
-        <v>660</v>
+        <v>668</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9126,13 +9205,13 @@
         <v>19</v>
       </c>
       <c r="B20" s="17" t="s">
-        <v>661</v>
+        <v>669</v>
       </c>
       <c r="C20" s="17" t="s">
-        <v>619</v>
+        <v>627</v>
       </c>
       <c r="D20" s="21" t="s">
-        <v>662</v>
+        <v>670</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9140,13 +9219,13 @@
         <v>20</v>
       </c>
       <c r="B21" s="17" t="s">
-        <v>663</v>
+        <v>671</v>
       </c>
       <c r="C21" s="17" t="s">
-        <v>664</v>
+        <v>672</v>
       </c>
       <c r="D21" s="21" t="s">
-        <v>665</v>
+        <v>673</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9154,14 +9233,26 @@
         <v>21</v>
       </c>
       <c r="B22" s="17" t="s">
-        <v>666</v>
+        <v>674</v>
       </c>
       <c r="C22" s="17" t="s">
-        <v>667</v>
+        <v>675</v>
       </c>
       <c r="D22" s="21" t="s">
-        <v>668</v>
-      </c>
+        <v>676</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="17" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="17" t="s">
+        <v>677</v>
+      </c>
+      <c r="C23" s="17" t="s">
+        <v>678</v>
+      </c>
+      <c r="D23" s="21"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Lens About: origin card, full marathon
Clicking "Grant" at the centre of About opens a small card:
- a headshot slot, a dashed placeholder until the photo arrives;
- two plain sentences on who Grant is and what he does now, as a
  draft, facts only;
- email and LinkedIn, from `site` in src/content.js.

It sits beside the centre on wide screens and is centred on phones. It
closes with ×, Esc or a click outside, and only shows in About. The
centre lights up on hover or focus, and About's hint mentions it.

LinkedIn (linkedin.com/in/grant-t-sacco) is added to the site's links,
so the "Get in touch" card shows it too. The email row reads "to add"
until Grant picks an address; the repo is public, so the workbook asks
which one to show.

The Austin Marathon is marked as the full 26.2 in its hover caption,
the workbook and CLAUDE.md.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KQRhL2ffDZuAUo4d7ziJty
</commit_message>
<xml_diff>
--- a/planning/site-artifacts.xlsx
+++ b/planning/site-artifacts.xlsx
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1532" uniqueCount="694">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1535" uniqueCount="697">
   <si>
     <t xml:space="preserve">Site artifacts: mapping workbook</t>
   </si>
@@ -1954,7 +1954,7 @@
     <t xml:space="preserve">Austin Marathon</t>
   </si>
   <si>
-    <t xml:space="preserve">February 2024. Its logo, small, on the 2024 ring in About (name on hover).</t>
+    <t xml:space="preserve">Full marathon (26.2 mi), February 2024. Its logo, small, on the 2024 ring in About (name on hover).</t>
   </si>
   <si>
     <t xml:space="preserve">Your note</t>
@@ -2150,6 +2150,15 @@
   </si>
   <si>
     <t xml:space="preserve">Races: was the Austin Marathon the full 26.2 or the half? Which month was IRONMAN 70.3 Texas (April is the placeholder)?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Austin Marathon: the full 26.2. IRONMAN month still open (April placeholder).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Origin card (click "Grant" in About): which email should it show? (The repo is public, so the address will be visible to scrapers; a forwarding address is an option.) Also: send the headshot, and edit the two draft sentences if you like.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">About, contact</t>
   </si>
 </sst>
 </file>
@@ -9008,7 +9017,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4"/>
@@ -9359,7 +9368,21 @@
       <c r="C25" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="D25" s="21"/>
+      <c r="D25" s="21" t="s">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="17" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="17" t="s">
+        <v>695</v>
+      </c>
+      <c r="C26" s="17" t="s">
+        <v>696</v>
+      </c>
+      <c r="D26" s="21"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Photos for the dry mix plant and the static mixer
- Dry mix plant: the Houston silo tower and the plant interior in its photo
  viewer.
- In-line static mixing: the mixer as installed and its piping drawing.
- All four from the portfolio; the site development stays as it is.
- Workbook updated (open question 35 answered).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KQRhL2ffDZuAUo4d7ziJty
</commit_message>
<xml_diff>
--- a/planning/site-artifacts.xlsx
+++ b/planning/site-artifacts.xlsx
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1560" uniqueCount="728">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1561" uniqueCount="729">
   <si>
     <t xml:space="preserve">Site artifacts: mapping workbook</t>
   </si>
@@ -532,7 +532,7 @@
     <t xml:space="preserve">Yes (Grant's exterior model of MAPEI Houston, v12)</t>
   </si>
   <si>
-    <t xml:space="preserve">Portfolio p.4: elevation, P&amp;ID, 3D render, tower photo, interior photo. MAPEI Houston exterior model (GLB v12) live in Lens v2 (zones: silo &amp; mixing tower, production &amp; warehouse, offices, site), opens with the tower lit; tile still + About hover turntable</t>
+    <t xml:space="preserve">Portfolio p.4: elevation, P&amp;ID, 3D render, tower photo, interior photo. MAPEI Houston exterior model (GLB v12) live in Lens v2 (zones: silo &amp; mixing tower, production &amp; warehouse, offices, site), opens with the tower lit; tile still + About hover turntable; photo viewer: the Houston silo tower and the plant interior (portfolio p.4)</t>
   </si>
   <si>
     <t xml:space="preserve">Dates: placeholder for now (About shows it at ~March 2022).</t>
@@ -625,7 +625,7 @@
     <t xml:space="preserve">Have CAD (render in portfolio)</t>
   </si>
   <si>
-    <t xml:space="preserve">Portfolio p.5: drawing, 3D render, photo</t>
+    <t xml:space="preserve">Photo viewer: the static mixer as installed and its piping drawing (portfolio p.5). Picture still a placeholder.</t>
   </si>
   <si>
     <t xml:space="preserve">E7</t>
@@ -2252,6 +2252,9 @@
   </si>
   <si>
     <t xml:space="preserve">E3, E4, E5, E6, photos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes: dry mix plant (tower and interior photos) and static mixing (mixer photo and piping drawing). Site development stays as it is.</t>
   </si>
 </sst>
 </file>
@@ -9605,7 +9608,9 @@
       <c r="C36" s="17" t="s">
         <v>727</v>
       </c>
-      <c r="D36" s="21"/>
+      <c r="D36" s="21" t="s">
+        <v>728</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Static mixer picture; CAD views for the dry mix plant
- In-line static mixing: the CAD render of the mixing skid (the larger
  portfolio copy) is its picture, trimmed and framed 3:2 on its own light
  blue background so the tall skid is not cropped.
- Dry mix plant: the silo tower in CAD (portfolio copy, larger than the one
  sent) and the plant's steel structure in CAD join its photo viewer, after
  the tower and interior photos (four in all).
- CLAUDE.md and the workbook updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KQRhL2ffDZuAUo4d7ziJty
</commit_message>
<xml_diff>
--- a/planning/site-artifacts.xlsx
+++ b/planning/site-artifacts.xlsx
@@ -532,7 +532,7 @@
     <t xml:space="preserve">Yes (Grant's exterior model of MAPEI Houston, v12)</t>
   </si>
   <si>
-    <t xml:space="preserve">Portfolio p.4: elevation, P&amp;ID, 3D render, tower photo, interior photo. MAPEI Houston exterior model (GLB v12) live in Lens v2 (zones: silo &amp; mixing tower, production &amp; warehouse, offices, site), opens with the tower lit; tile still + About hover turntable; photo viewer: the Houston silo tower and the plant interior (portfolio p.4)</t>
+    <t xml:space="preserve">Portfolio p.4: elevation, P&amp;ID, 3D render, tower photo, interior photo. MAPEI Houston exterior model (GLB v12) live in Lens v2 (zones: silo &amp; mixing tower, production &amp; warehouse, offices, site), opens with the tower lit; tile still + About hover turntable; photo viewer: the Houston silo tower and plant interior photos, the tower in CAD (portfolio p.4) and the plant structure in CAD (sent by Grant)</t>
   </si>
   <si>
     <t xml:space="preserve">Dates: placeholder for now (About shows it at ~March 2022).</t>
@@ -625,7 +625,7 @@
     <t xml:space="preserve">Have CAD (render in portfolio)</t>
   </si>
   <si>
-    <t xml:space="preserve">Photo viewer: the static mixer as installed and its piping drawing (portfolio p.5). Picture still a placeholder.</t>
+    <t xml:space="preserve">Cover picture: CAD render of the mixing skid (portfolio p.5), framed 3:2; photo viewer: the static mixer as installed and its piping drawing (portfolio p.5)</t>
   </si>
   <si>
     <t xml:space="preserve">E7</t>

</xml_diff>

<commit_message>
Record the MPOC decision: keep the plain blocks
Grant chose to keep the MPOC as plain blocks rather than build the detailed
layout from his Pascal file (the real floor plan). Workbook question 29 and
CLAUDE.md updated; no site change.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KQRhL2ffDZuAUo4d7ziJty
</commit_message>
<xml_diff>
--- a/planning/site-artifacts.xlsx
+++ b/planning/site-artifacts.xlsx
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1561" uniqueCount="729">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1562" uniqueCount="730">
   <si>
     <t xml:space="preserve">Site artifacts: mapping workbook</t>
   </si>
@@ -2213,6 +2213,9 @@
   </si>
   <si>
     <t xml:space="preserve">E1, E2, 3D model</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keep plain blocks (no detailed layout on the public site).</t>
   </si>
   <si>
     <t xml:space="preserve">MPOC: where is the additive &amp; subtractive manufacturing lab? It is placed at the east end, behind the offices, as a guess.</t>
@@ -9534,17 +9537,19 @@
       <c r="C30" s="17" t="s">
         <v>714</v>
       </c>
-      <c r="D30" s="21"/>
+      <c r="D30" s="21" t="s">
+        <v>715</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="17" t="n">
         <v>30</v>
       </c>
       <c r="B31" s="17" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="C31" s="17" t="s">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="D31" s="21"/>
     </row>
@@ -9553,10 +9558,10 @@
         <v>31</v>
       </c>
       <c r="B32" s="17" t="s">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="C32" s="17" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="D32" s="21"/>
     </row>
@@ -9565,10 +9570,10 @@
         <v>32</v>
       </c>
       <c r="B33" s="17" t="s">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="C33" s="17" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="D33" s="21"/>
     </row>
@@ -9577,10 +9582,10 @@
         <v>33</v>
       </c>
       <c r="B34" s="17" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="C34" s="17" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="D34" s="21"/>
     </row>
@@ -9589,13 +9594,13 @@
         <v>34</v>
       </c>
       <c r="B35" s="17" t="s">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="C35" s="17" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="D35" s="21" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9603,13 +9608,13 @@
         <v>35</v>
       </c>
       <c r="B36" s="17" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="C36" s="17" t="s">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="D36" s="21" t="s">
-        <v>728</v>
+        <v>729</v>
       </c>
     </row>
   </sheetData>

</xml_diff>